<commit_message>
v83: add 2026-10-27 exit polls to channel polls
סקרים לפי ערוץ now holds the latest exit poll from each of the six
channels that published one (Channel 12, 13, Kan, 14, i24, 16), each
summing to 120 seats; חישוב לפי ערוץ is rebuilt for them. Each poll's
date cell carries a comment naming its source.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C84BdUz8Pbr2phmrWK39vV
</commit_message>
<xml_diff>
--- a/party-comparison-updated-v83.xlsx
+++ b/party-comparison-updated-v83.xlsx
@@ -311,8 +311,178 @@
 </comments>
 </file>
 
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="B2" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">מדגם מעודכן</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">. Maariv 28/10/2026 02:19 (maariv.co.il/news/elections-2026/article-1382036); </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">המשותפת </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">12 לפי סך הגוש הערבי (19) בכתבה</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B3" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">מדגם מעודכן</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">. Maariv 28/10/2026 02:19 (maariv.co.il/news/elections-2026/article-1382036); </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">המשותפת </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">11 לפי סך הגוש הערבי (18) בכתבה</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">מדגם מעודכן </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">01:43. maariv.co.il/breaking-news/article-1382115 + </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">מדגם ראשון ב</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">-ynet</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">מדגם מעודכן (גוש נתניהו </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">62). Maariv 28/10/2026 02:19 (maariv.co.il/news/elections-2026/article-1382036); ynet.co.il/news/article/h1nq00srhme</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Maariv 28/10/2026 02:19 (maariv.co.il/news/elections-2026/article-1382036)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">מדגם ראשון (אין עדכון)</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">. ynet.co.il/news/elections2026/article/rks5sp03zx</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7380" uniqueCount="1834">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7554" uniqueCount="1852">
   <si>
     <t xml:space="preserve">מפלגה</t>
   </si>
@@ -7072,6 +7242,117 @@
     <t xml:space="preserve">מספר משיבים</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">חדשות </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מנו גבע</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">חדשות </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">13</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">המדד</t>
+  </si>
+  <si>
+    <t xml:space="preserve">כאן חדשות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">דודי חסיד</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ערוץ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">שלמה פילבר</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i24 news</t>
+  </si>
+  <si>
+    <t xml:space="preserve">צוריאל שרון</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ערוץ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">יצחק כ״ץ</t>
+  </si>
+  <si>
     <t xml:space="preserve">מנדטים</t>
   </si>
   <si>
@@ -7135,6 +7416,176 @@
   </si>
   <si>
     <t xml:space="preserve">הערה</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ש</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ס</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">רע</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">מ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ביחד </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">בנט</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">לפיד</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ישר</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">!</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">המילואימניקים</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">הכלכלית</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -47126,12 +47577,324 @@
         <v>1497</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>1832</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>1833</v>
+      </c>
+      <c r="E2" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I2" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="J2" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="K2" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="M2" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="N2" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="O2" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="P2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>1832</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>1835</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="I3" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="J3" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="K3" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="L3" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="M3" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="N3" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="O3" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="P3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>1832</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>1837</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="I4" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="K4" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="M4" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="N4" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="O4" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="P4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>1832</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>1839</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="I5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="K5" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="L5" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="M5" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="N5" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="O5" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>1832</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>1841</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="I6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="K6" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="M6" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="N6" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="O6" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="P6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>1832</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>1843</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="G7" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="H7" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="I7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="K7" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="L7" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="M7" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="N7" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="O7" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="P7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -47140,6 +47903,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -47148,7 +47912,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr defaultColWidth="8.53125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -47162,7 +47926,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>1831</v>
+        <v>1844</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>1472</v>
@@ -47174,10 +47938,2818 @@
         <v>1807</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>1832</v>
+        <v>1845</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>1833</v>
+        <v>1846</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B2" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A2,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A2,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>27</v>
+      </c>
+      <c r="E2" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C2,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D2)</f>
+        <v>4</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C2,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D2)</f>
+        <v>23</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <f aca="false">IF($D2=0,0,$E2/$D2)</f>
+        <v>0.148148148148148</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C2)</f>
+        <v>36</v>
+      </c>
+      <c r="I2" s="0" t="str">
+        <f aca="false">IF(AND($D2&gt;0,$H2=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B3" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A3,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>1480</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A3,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C3,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D3)</f>
+        <v>0</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C3,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D3)</f>
+        <v>6</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <f aca="false">IF($D3=0,0,$E3/$D3)</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C3)</f>
+        <v>9</v>
+      </c>
+      <c r="I3" s="0" t="str">
+        <f aca="false">IF(AND($D3&gt;0,$H3=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B4" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A4,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>1847</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A4,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C4,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D4)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C4,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D4)</f>
+        <v>7</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <f aca="false">IF($D4=0,0,$E4/$D4)</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C4)</f>
+        <v>11</v>
+      </c>
+      <c r="I4" s="0" t="str">
+        <f aca="false">IF(AND($D4&gt;0,$H4=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B5" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A5,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A5,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>12</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C5,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D5)</f>
+        <v>2</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C5,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D5)</f>
+        <v>8</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <f aca="false">IF($D5=0,0,$E5/$D5)</f>
+        <v>0.166666666666667</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C5)</f>
+        <v>10</v>
+      </c>
+      <c r="I5" s="0" t="str">
+        <f aca="false">IF(AND($D5&gt;0,$H5=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B6" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A6,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A6,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C6,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D6)</f>
+        <v>2</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C6,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D6)</f>
+        <v>5</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <f aca="false">IF($D6=0,0,$E6/$D6)</f>
+        <v>0.285714285714286</v>
+      </c>
+      <c r="H6" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C6)</f>
+        <v>20</v>
+      </c>
+      <c r="I6" s="0" t="str">
+        <f aca="false">IF(AND($D6&gt;0,$H6=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B7" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A7,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A7,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>9</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C7,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D7)</f>
+        <v>4</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C7,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D7)</f>
+        <v>5</v>
+      </c>
+      <c r="G7" s="0" t="n">
+        <f aca="false">IF($D7=0,0,$E7/$D7)</f>
+        <v>0.444444444444444</v>
+      </c>
+      <c r="H7" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C7)</f>
+        <v>20</v>
+      </c>
+      <c r="I7" s="0" t="str">
+        <f aca="false">IF(AND($D7&gt;0,$H7=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B8" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A8,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A8,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C8,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D8)</f>
+        <v>1</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C8,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D8)</f>
+        <v>5</v>
+      </c>
+      <c r="G8" s="0" t="n">
+        <f aca="false">IF($D8=0,0,$E8/$D8)</f>
+        <v>0.166666666666667</v>
+      </c>
+      <c r="H8" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C8)</f>
+        <v>18</v>
+      </c>
+      <c r="I8" s="0" t="str">
+        <f aca="false">IF(AND($D8&gt;0,$H8=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B9" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A9,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>1848</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A9,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C9,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D9)</f>
+        <v>1</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C9,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D9)</f>
+        <v>5</v>
+      </c>
+      <c r="G9" s="0" t="n">
+        <f aca="false">IF($D9=0,0,$E9/$D9)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H9" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C9)</f>
+        <v>6</v>
+      </c>
+      <c r="I9" s="0" t="str">
+        <f aca="false">IF(AND($D9&gt;0,$H9=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B10" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A10,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A10,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C10,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D10)</f>
+        <v>2</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C10,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D10)</f>
+        <v>4</v>
+      </c>
+      <c r="G10" s="0" t="n">
+        <f aca="false">IF($D10=0,0,$E10/$D10)</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="H10" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C10)</f>
+        <v>17</v>
+      </c>
+      <c r="I10" s="0" t="str">
+        <f aca="false">IF(AND($D10&gt;0,$H10=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B11" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A11,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A11,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>12</v>
+      </c>
+      <c r="E11" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C11,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D11)</f>
+        <v>6</v>
+      </c>
+      <c r="F11" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C11,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D11)</f>
+        <v>6</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <f aca="false">IF($D11=0,0,$E11/$D11)</f>
+        <v>0.5</v>
+      </c>
+      <c r="H11" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C11)</f>
+        <v>26</v>
+      </c>
+      <c r="I11" s="0" t="str">
+        <f aca="false">IF(AND($D11&gt;0,$H11=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B12" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A12,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D12" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A12,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>21</v>
+      </c>
+      <c r="E12" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C12,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D12)</f>
+        <v>11</v>
+      </c>
+      <c r="F12" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C12,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D12)</f>
+        <v>10</v>
+      </c>
+      <c r="G12" s="0" t="n">
+        <f aca="false">IF($D12=0,0,$E12/$D12)</f>
+        <v>0.523809523809524</v>
+      </c>
+      <c r="H12" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C12)</f>
+        <v>40</v>
+      </c>
+      <c r="I12" s="0" t="str">
+        <f aca="false">IF(AND($D12&gt;0,$H12=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B13" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A13,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A13,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C13,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D13)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C13,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D13)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="0" t="n">
+        <f aca="false">IF($D13=0,0,$E13/$D13)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C13)</f>
+        <v>11</v>
+      </c>
+      <c r="I13" s="0" t="str">
+        <f aca="false">IF(AND($D13&gt;0,$H13=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B14" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A14,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A14,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C14,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D14)</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C14,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D14)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="0" t="n">
+        <f aca="false">IF($D14=0,0,$E14/$D14)</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C14)</f>
+        <v>20</v>
+      </c>
+      <c r="I14" s="0" t="str">
+        <f aca="false">IF(AND($D14&gt;0,$H14=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B15" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A15,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D15" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A15,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>27</v>
+      </c>
+      <c r="E15" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C15,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D15)</f>
+        <v>4</v>
+      </c>
+      <c r="F15" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C15,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D15)</f>
+        <v>23</v>
+      </c>
+      <c r="G15" s="0" t="n">
+        <f aca="false">IF($D15=0,0,$E15/$D15)</f>
+        <v>0.148148148148148</v>
+      </c>
+      <c r="H15" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C15)</f>
+        <v>36</v>
+      </c>
+      <c r="I15" s="0" t="str">
+        <f aca="false">IF(AND($D15&gt;0,$H15=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B16" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A16,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>1480</v>
+      </c>
+      <c r="D16" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A16,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E16" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C16,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D16)</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C16,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D16)</f>
+        <v>6</v>
+      </c>
+      <c r="G16" s="0" t="n">
+        <f aca="false">IF($D16=0,0,$E16/$D16)</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C16)</f>
+        <v>9</v>
+      </c>
+      <c r="I16" s="0" t="str">
+        <f aca="false">IF(AND($D16&gt;0,$H16=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B17" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A17,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>1847</v>
+      </c>
+      <c r="D17" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A17,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E17" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C17,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D17)</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C17,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D17)</f>
+        <v>6</v>
+      </c>
+      <c r="G17" s="0" t="n">
+        <f aca="false">IF($D17=0,0,$E17/$D17)</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C17)</f>
+        <v>11</v>
+      </c>
+      <c r="I17" s="0" t="str">
+        <f aca="false">IF(AND($D17&gt;0,$H17=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B18" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A18,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D18" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A18,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>11</v>
+      </c>
+      <c r="E18" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C18,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D18)</f>
+        <v>2</v>
+      </c>
+      <c r="F18" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C18,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D18)</f>
+        <v>8</v>
+      </c>
+      <c r="G18" s="0" t="n">
+        <f aca="false">IF($D18=0,0,$E18/$D18)</f>
+        <v>0.181818181818182</v>
+      </c>
+      <c r="H18" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C18)</f>
+        <v>10</v>
+      </c>
+      <c r="I18" s="0" t="str">
+        <f aca="false">IF(AND($D18&gt;0,$H18=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B19" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A19,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D19" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A19,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E19" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C19,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D19)</f>
+        <v>2</v>
+      </c>
+      <c r="F19" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C19,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D19)</f>
+        <v>5</v>
+      </c>
+      <c r="G19" s="0" t="n">
+        <f aca="false">IF($D19=0,0,$E19/$D19)</f>
+        <v>0.285714285714286</v>
+      </c>
+      <c r="H19" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C19)</f>
+        <v>20</v>
+      </c>
+      <c r="I19" s="0" t="str">
+        <f aca="false">IF(AND($D19&gt;0,$H19=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B20" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A20,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D20" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A20,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>9</v>
+      </c>
+      <c r="E20" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C20,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D20)</f>
+        <v>4</v>
+      </c>
+      <c r="F20" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C20,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D20)</f>
+        <v>5</v>
+      </c>
+      <c r="G20" s="0" t="n">
+        <f aca="false">IF($D20=0,0,$E20/$D20)</f>
+        <v>0.444444444444444</v>
+      </c>
+      <c r="H20" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C20)</f>
+        <v>20</v>
+      </c>
+      <c r="I20" s="0" t="str">
+        <f aca="false">IF(AND($D20&gt;0,$H20=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B21" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A21,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A21,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E21" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C21,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D21)</f>
+        <v>1</v>
+      </c>
+      <c r="F21" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C21,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D21)</f>
+        <v>5</v>
+      </c>
+      <c r="G21" s="0" t="n">
+        <f aca="false">IF($D21=0,0,$E21/$D21)</f>
+        <v>0.166666666666667</v>
+      </c>
+      <c r="H21" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C21)</f>
+        <v>18</v>
+      </c>
+      <c r="I21" s="0" t="str">
+        <f aca="false">IF(AND($D21&gt;0,$H21=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B22" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A22,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>1848</v>
+      </c>
+      <c r="D22" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A22,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E22" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C22,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D22)</f>
+        <v>1</v>
+      </c>
+      <c r="F22" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C22,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D22)</f>
+        <v>5</v>
+      </c>
+      <c r="G22" s="0" t="n">
+        <f aca="false">IF($D22=0,0,$E22/$D22)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H22" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C22)</f>
+        <v>6</v>
+      </c>
+      <c r="I22" s="0" t="str">
+        <f aca="false">IF(AND($D22&gt;0,$H22=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B23" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A23,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D23" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A23,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E23" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C23,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D23)</f>
+        <v>2</v>
+      </c>
+      <c r="F23" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C23,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D23)</f>
+        <v>4</v>
+      </c>
+      <c r="G23" s="0" t="n">
+        <f aca="false">IF($D23=0,0,$E23/$D23)</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="H23" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C23)</f>
+        <v>17</v>
+      </c>
+      <c r="I23" s="0" t="str">
+        <f aca="false">IF(AND($D23&gt;0,$H23=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B24" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A24,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="D24" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A24,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>13</v>
+      </c>
+      <c r="E24" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C24,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D24)</f>
+        <v>6</v>
+      </c>
+      <c r="F24" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C24,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D24)</f>
+        <v>7</v>
+      </c>
+      <c r="G24" s="0" t="n">
+        <f aca="false">IF($D24=0,0,$E24/$D24)</f>
+        <v>0.461538461538462</v>
+      </c>
+      <c r="H24" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C24)</f>
+        <v>26</v>
+      </c>
+      <c r="I24" s="0" t="str">
+        <f aca="false">IF(AND($D24&gt;0,$H24=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B25" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A25,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D25" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A25,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>22</v>
+      </c>
+      <c r="E25" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C25,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D25)</f>
+        <v>11</v>
+      </c>
+      <c r="F25" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C25,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D25)</f>
+        <v>11</v>
+      </c>
+      <c r="G25" s="0" t="n">
+        <f aca="false">IF($D25=0,0,$E25/$D25)</f>
+        <v>0.5</v>
+      </c>
+      <c r="H25" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C25)</f>
+        <v>40</v>
+      </c>
+      <c r="I25" s="0" t="str">
+        <f aca="false">IF(AND($D25&gt;0,$H25=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B26" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A26,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="D26" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A26,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C26,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D26)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C26,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D26)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="0" t="n">
+        <f aca="false">IF($D26=0,0,$E26/$D26)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C26)</f>
+        <v>11</v>
+      </c>
+      <c r="I26" s="0" t="str">
+        <f aca="false">IF(AND($D26&gt;0,$H26=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B27" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A27,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D27" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A27,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C27,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D27)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C27,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D27)</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="0" t="n">
+        <f aca="false">IF($D27=0,0,$E27/$D27)</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C27)</f>
+        <v>20</v>
+      </c>
+      <c r="I27" s="0" t="str">
+        <f aca="false">IF(AND($D27&gt;0,$H27=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B28" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A28,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D28" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A28,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>27</v>
+      </c>
+      <c r="E28" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C28,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D28)</f>
+        <v>4</v>
+      </c>
+      <c r="F28" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C28,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D28)</f>
+        <v>23</v>
+      </c>
+      <c r="G28" s="0" t="n">
+        <f aca="false">IF($D28=0,0,$E28/$D28)</f>
+        <v>0.148148148148148</v>
+      </c>
+      <c r="H28" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C28)</f>
+        <v>36</v>
+      </c>
+      <c r="I28" s="0" t="str">
+        <f aca="false">IF(AND($D28&gt;0,$H28=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B29" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A29,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>1480</v>
+      </c>
+      <c r="D29" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A29,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E29" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C29,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D29)</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C29,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D29)</f>
+        <v>6</v>
+      </c>
+      <c r="G29" s="0" t="n">
+        <f aca="false">IF($D29=0,0,$E29/$D29)</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C29)</f>
+        <v>9</v>
+      </c>
+      <c r="I29" s="0" t="str">
+        <f aca="false">IF(AND($D29&gt;0,$H29=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B30" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A30,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>1847</v>
+      </c>
+      <c r="D30" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A30,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E30" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C30,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D30)</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C30,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D30)</f>
+        <v>6</v>
+      </c>
+      <c r="G30" s="0" t="n">
+        <f aca="false">IF($D30=0,0,$E30/$D30)</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C30)</f>
+        <v>11</v>
+      </c>
+      <c r="I30" s="0" t="str">
+        <f aca="false">IF(AND($D30&gt;0,$H30=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B31" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A31,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D31" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A31,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>11</v>
+      </c>
+      <c r="E31" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C31,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D31)</f>
+        <v>2</v>
+      </c>
+      <c r="F31" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C31,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D31)</f>
+        <v>8</v>
+      </c>
+      <c r="G31" s="0" t="n">
+        <f aca="false">IF($D31=0,0,$E31/$D31)</f>
+        <v>0.181818181818182</v>
+      </c>
+      <c r="H31" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C31)</f>
+        <v>10</v>
+      </c>
+      <c r="I31" s="0" t="str">
+        <f aca="false">IF(AND($D31&gt;0,$H31=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B32" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A32,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D32" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A32,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>8</v>
+      </c>
+      <c r="E32" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C32,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D32)</f>
+        <v>2</v>
+      </c>
+      <c r="F32" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C32,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D32)</f>
+        <v>6</v>
+      </c>
+      <c r="G32" s="0" t="n">
+        <f aca="false">IF($D32=0,0,$E32/$D32)</f>
+        <v>0.25</v>
+      </c>
+      <c r="H32" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C32)</f>
+        <v>20</v>
+      </c>
+      <c r="I32" s="0" t="str">
+        <f aca="false">IF(AND($D32&gt;0,$H32=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B33" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A33,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D33" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A33,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>9</v>
+      </c>
+      <c r="E33" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C33,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D33)</f>
+        <v>4</v>
+      </c>
+      <c r="F33" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C33,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D33)</f>
+        <v>5</v>
+      </c>
+      <c r="G33" s="0" t="n">
+        <f aca="false">IF($D33=0,0,$E33/$D33)</f>
+        <v>0.444444444444444</v>
+      </c>
+      <c r="H33" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C33)</f>
+        <v>20</v>
+      </c>
+      <c r="I33" s="0" t="str">
+        <f aca="false">IF(AND($D33&gt;0,$H33=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B34" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A34,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D34" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A34,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E34" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C34,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D34)</f>
+        <v>1</v>
+      </c>
+      <c r="F34" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C34,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D34)</f>
+        <v>5</v>
+      </c>
+      <c r="G34" s="0" t="n">
+        <f aca="false">IF($D34=0,0,$E34/$D34)</f>
+        <v>0.166666666666667</v>
+      </c>
+      <c r="H34" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C34)</f>
+        <v>18</v>
+      </c>
+      <c r="I34" s="0" t="str">
+        <f aca="false">IF(AND($D34&gt;0,$H34=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B35" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A35,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>1848</v>
+      </c>
+      <c r="D35" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A35,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E35" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C35,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D35)</f>
+        <v>1</v>
+      </c>
+      <c r="F35" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C35,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D35)</f>
+        <v>5</v>
+      </c>
+      <c r="G35" s="0" t="n">
+        <f aca="false">IF($D35=0,0,$E35/$D35)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H35" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C35)</f>
+        <v>6</v>
+      </c>
+      <c r="I35" s="0" t="str">
+        <f aca="false">IF(AND($D35&gt;0,$H35=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B36" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A36,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D36" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A36,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E36" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C36,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D36)</f>
+        <v>2</v>
+      </c>
+      <c r="F36" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C36,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D36)</f>
+        <v>4</v>
+      </c>
+      <c r="G36" s="0" t="n">
+        <f aca="false">IF($D36=0,0,$E36/$D36)</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="H36" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C36)</f>
+        <v>17</v>
+      </c>
+      <c r="I36" s="0" t="str">
+        <f aca="false">IF(AND($D36&gt;0,$H36=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B37" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A37,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="D37" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A37,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>13</v>
+      </c>
+      <c r="E37" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C37,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D37)</f>
+        <v>6</v>
+      </c>
+      <c r="F37" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C37,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D37)</f>
+        <v>7</v>
+      </c>
+      <c r="G37" s="0" t="n">
+        <f aca="false">IF($D37=0,0,$E37/$D37)</f>
+        <v>0.461538461538462</v>
+      </c>
+      <c r="H37" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C37)</f>
+        <v>26</v>
+      </c>
+      <c r="I37" s="0" t="str">
+        <f aca="false">IF(AND($D37&gt;0,$H37=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B38" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A38,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D38" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A38,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>21</v>
+      </c>
+      <c r="E38" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C38,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D38)</f>
+        <v>11</v>
+      </c>
+      <c r="F38" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C38,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D38)</f>
+        <v>10</v>
+      </c>
+      <c r="G38" s="0" t="n">
+        <f aca="false">IF($D38=0,0,$E38/$D38)</f>
+        <v>0.523809523809524</v>
+      </c>
+      <c r="H38" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C38)</f>
+        <v>40</v>
+      </c>
+      <c r="I38" s="0" t="str">
+        <f aca="false">IF(AND($D38&gt;0,$H38=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B39" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A39,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="D39" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A39,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C39,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D39)</f>
+        <v>0</v>
+      </c>
+      <c r="F39" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C39,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D39)</f>
+        <v>0</v>
+      </c>
+      <c r="G39" s="0" t="n">
+        <f aca="false">IF($D39=0,0,$E39/$D39)</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C39)</f>
+        <v>11</v>
+      </c>
+      <c r="I39" s="0" t="str">
+        <f aca="false">IF(AND($D39&gt;0,$H39=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B40" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A40,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D40" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A40,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C40,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D40)</f>
+        <v>0</v>
+      </c>
+      <c r="F40" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C40,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D40)</f>
+        <v>0</v>
+      </c>
+      <c r="G40" s="0" t="n">
+        <f aca="false">IF($D40=0,0,$E40/$D40)</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C40)</f>
+        <v>20</v>
+      </c>
+      <c r="I40" s="0" t="str">
+        <f aca="false">IF(AND($D40&gt;0,$H40=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B41" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A41,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D41" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A41,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>31</v>
+      </c>
+      <c r="E41" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C41,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D41)</f>
+        <v>4</v>
+      </c>
+      <c r="F41" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C41,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D41)</f>
+        <v>27</v>
+      </c>
+      <c r="G41" s="0" t="n">
+        <f aca="false">IF($D41=0,0,$E41/$D41)</f>
+        <v>0.129032258064516</v>
+      </c>
+      <c r="H41" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C41)</f>
+        <v>36</v>
+      </c>
+      <c r="I41" s="0" t="str">
+        <f aca="false">IF(AND($D41&gt;0,$H41=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B42" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A42,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>1480</v>
+      </c>
+      <c r="D42" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A42,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E42" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C42,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D42)</f>
+        <v>0</v>
+      </c>
+      <c r="F42" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C42,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D42)</f>
+        <v>7</v>
+      </c>
+      <c r="G42" s="0" t="n">
+        <f aca="false">IF($D42=0,0,$E42/$D42)</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C42)</f>
+        <v>9</v>
+      </c>
+      <c r="I42" s="0" t="str">
+        <f aca="false">IF(AND($D42&gt;0,$H42=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B43" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A43,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>1847</v>
+      </c>
+      <c r="D43" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A43,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>10</v>
+      </c>
+      <c r="E43" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C43,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D43)</f>
+        <v>0</v>
+      </c>
+      <c r="F43" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C43,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D43)</f>
+        <v>10</v>
+      </c>
+      <c r="G43" s="0" t="n">
+        <f aca="false">IF($D43=0,0,$E43/$D43)</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C43)</f>
+        <v>11</v>
+      </c>
+      <c r="I43" s="0" t="str">
+        <f aca="false">IF(AND($D43&gt;0,$H43=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B44" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A44,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D44" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A44,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>11</v>
+      </c>
+      <c r="E44" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C44,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D44)</f>
+        <v>2</v>
+      </c>
+      <c r="F44" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C44,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D44)</f>
+        <v>8</v>
+      </c>
+      <c r="G44" s="0" t="n">
+        <f aca="false">IF($D44=0,0,$E44/$D44)</f>
+        <v>0.181818181818182</v>
+      </c>
+      <c r="H44" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C44)</f>
+        <v>10</v>
+      </c>
+      <c r="I44" s="0" t="str">
+        <f aca="false">IF(AND($D44&gt;0,$H44=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B45" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A45,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A45,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E45" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C45,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D45)</f>
+        <v>0</v>
+      </c>
+      <c r="F45" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C45,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D45)</f>
+        <v>0</v>
+      </c>
+      <c r="G45" s="0" t="n">
+        <f aca="false">IF($D45=0,0,$E45/$D45)</f>
+        <v>0</v>
+      </c>
+      <c r="H45" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C45)</f>
+        <v>20</v>
+      </c>
+      <c r="I45" s="0" t="str">
+        <f aca="false">IF(AND($D45&gt;0,$H45=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B46" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A46,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C46" s="13" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D46" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A46,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>9</v>
+      </c>
+      <c r="E46" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C46,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D46)</f>
+        <v>4</v>
+      </c>
+      <c r="F46" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C46,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D46)</f>
+        <v>5</v>
+      </c>
+      <c r="G46" s="0" t="n">
+        <f aca="false">IF($D46=0,0,$E46/$D46)</f>
+        <v>0.444444444444444</v>
+      </c>
+      <c r="H46" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C46)</f>
+        <v>20</v>
+      </c>
+      <c r="I46" s="0" t="str">
+        <f aca="false">IF(AND($D46&gt;0,$H46=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B47" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A47,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C47" s="13" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D47" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A47,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E47" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C47,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D47)</f>
+        <v>1</v>
+      </c>
+      <c r="F47" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C47,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D47)</f>
+        <v>6</v>
+      </c>
+      <c r="G47" s="0" t="n">
+        <f aca="false">IF($D47=0,0,$E47/$D47)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H47" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C47)</f>
+        <v>18</v>
+      </c>
+      <c r="I47" s="0" t="str">
+        <f aca="false">IF(AND($D47&gt;0,$H47=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B48" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A48,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C48" s="13" t="s">
+        <v>1848</v>
+      </c>
+      <c r="D48" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A48,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E48" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C48,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D48)</f>
+        <v>1</v>
+      </c>
+      <c r="F48" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C48,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D48)</f>
+        <v>5</v>
+      </c>
+      <c r="G48" s="0" t="n">
+        <f aca="false">IF($D48=0,0,$E48/$D48)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H48" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C48)</f>
+        <v>6</v>
+      </c>
+      <c r="I48" s="0" t="str">
+        <f aca="false">IF(AND($D48&gt;0,$H48=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B49" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A49,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D49" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A49,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E49" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C49,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D49)</f>
+        <v>2</v>
+      </c>
+      <c r="F49" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C49,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D49)</f>
+        <v>5</v>
+      </c>
+      <c r="G49" s="0" t="n">
+        <f aca="false">IF($D49=0,0,$E49/$D49)</f>
+        <v>0.285714285714286</v>
+      </c>
+      <c r="H49" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C49)</f>
+        <v>17</v>
+      </c>
+      <c r="I49" s="0" t="str">
+        <f aca="false">IF(AND($D49&gt;0,$H49=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B50" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A50,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C50" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="D50" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A50,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>11</v>
+      </c>
+      <c r="E50" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C50,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D50)</f>
+        <v>6</v>
+      </c>
+      <c r="F50" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C50,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D50)</f>
+        <v>5</v>
+      </c>
+      <c r="G50" s="0" t="n">
+        <f aca="false">IF($D50=0,0,$E50/$D50)</f>
+        <v>0.545454545454545</v>
+      </c>
+      <c r="H50" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C50)</f>
+        <v>26</v>
+      </c>
+      <c r="I50" s="0" t="str">
+        <f aca="false">IF(AND($D50&gt;0,$H50=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B51" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A51,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D51" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A51,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>20</v>
+      </c>
+      <c r="E51" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C51,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D51)</f>
+        <v>10</v>
+      </c>
+      <c r="F51" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C51,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D51)</f>
+        <v>10</v>
+      </c>
+      <c r="G51" s="0" t="n">
+        <f aca="false">IF($D51=0,0,$E51/$D51)</f>
+        <v>0.5</v>
+      </c>
+      <c r="H51" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C51)</f>
+        <v>40</v>
+      </c>
+      <c r="I51" s="0" t="str">
+        <f aca="false">IF(AND($D51&gt;0,$H51=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B52" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A52,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C52" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="D52" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A52,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E52" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C52,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D52)</f>
+        <v>0</v>
+      </c>
+      <c r="F52" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C52,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D52)</f>
+        <v>0</v>
+      </c>
+      <c r="G52" s="0" t="n">
+        <f aca="false">IF($D52=0,0,$E52/$D52)</f>
+        <v>0</v>
+      </c>
+      <c r="H52" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C52)</f>
+        <v>11</v>
+      </c>
+      <c r="I52" s="0" t="str">
+        <f aca="false">IF(AND($D52&gt;0,$H52=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="13" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B53" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A53,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C53" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D53" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A53,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E53" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C53,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D53)</f>
+        <v>0</v>
+      </c>
+      <c r="F53" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C53,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D53)</f>
+        <v>0</v>
+      </c>
+      <c r="G53" s="0" t="n">
+        <f aca="false">IF($D53=0,0,$E53/$D53)</f>
+        <v>0</v>
+      </c>
+      <c r="H53" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C53)</f>
+        <v>20</v>
+      </c>
+      <c r="I53" s="0" t="str">
+        <f aca="false">IF(AND($D53&gt;0,$H53=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B54" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A54,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D54" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A54,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>27</v>
+      </c>
+      <c r="E54" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C54,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D54)</f>
+        <v>4</v>
+      </c>
+      <c r="F54" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C54,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D54)</f>
+        <v>23</v>
+      </c>
+      <c r="G54" s="0" t="n">
+        <f aca="false">IF($D54=0,0,$E54/$D54)</f>
+        <v>0.148148148148148</v>
+      </c>
+      <c r="H54" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C54)</f>
+        <v>36</v>
+      </c>
+      <c r="I54" s="0" t="str">
+        <f aca="false">IF(AND($D54&gt;0,$H54=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B55" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A55,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C55" s="13" t="s">
+        <v>1480</v>
+      </c>
+      <c r="D55" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A55,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E55" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C55,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D55)</f>
+        <v>0</v>
+      </c>
+      <c r="F55" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C55,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D55)</f>
+        <v>7</v>
+      </c>
+      <c r="G55" s="0" t="n">
+        <f aca="false">IF($D55=0,0,$E55/$D55)</f>
+        <v>0</v>
+      </c>
+      <c r="H55" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C55)</f>
+        <v>9</v>
+      </c>
+      <c r="I55" s="0" t="str">
+        <f aca="false">IF(AND($D55&gt;0,$H55=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B56" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A56,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C56" s="13" t="s">
+        <v>1847</v>
+      </c>
+      <c r="D56" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A56,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>8</v>
+      </c>
+      <c r="E56" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C56,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D56)</f>
+        <v>0</v>
+      </c>
+      <c r="F56" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C56,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D56)</f>
+        <v>8</v>
+      </c>
+      <c r="G56" s="0" t="n">
+        <f aca="false">IF($D56=0,0,$E56/$D56)</f>
+        <v>0</v>
+      </c>
+      <c r="H56" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C56)</f>
+        <v>11</v>
+      </c>
+      <c r="I56" s="0" t="str">
+        <f aca="false">IF(AND($D56&gt;0,$H56=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B57" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A57,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C57" s="13" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D57" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A57,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>9</v>
+      </c>
+      <c r="E57" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C57,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D57)</f>
+        <v>2</v>
+      </c>
+      <c r="F57" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C57,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D57)</f>
+        <v>7</v>
+      </c>
+      <c r="G57" s="0" t="n">
+        <f aca="false">IF($D57=0,0,$E57/$D57)</f>
+        <v>0.222222222222222</v>
+      </c>
+      <c r="H57" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C57)</f>
+        <v>10</v>
+      </c>
+      <c r="I57" s="0" t="str">
+        <f aca="false">IF(AND($D57&gt;0,$H57=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B58" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A58,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D58" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A58,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>5</v>
+      </c>
+      <c r="E58" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C58,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D58)</f>
+        <v>2</v>
+      </c>
+      <c r="F58" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C58,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D58)</f>
+        <v>3</v>
+      </c>
+      <c r="G58" s="0" t="n">
+        <f aca="false">IF($D58=0,0,$E58/$D58)</f>
+        <v>0.4</v>
+      </c>
+      <c r="H58" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C58)</f>
+        <v>20</v>
+      </c>
+      <c r="I58" s="0" t="str">
+        <f aca="false">IF(AND($D58&gt;0,$H58=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B59" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A59,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C59" s="13" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D59" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A59,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>9</v>
+      </c>
+      <c r="E59" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C59,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D59)</f>
+        <v>4</v>
+      </c>
+      <c r="F59" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C59,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D59)</f>
+        <v>5</v>
+      </c>
+      <c r="G59" s="0" t="n">
+        <f aca="false">IF($D59=0,0,$E59/$D59)</f>
+        <v>0.444444444444444</v>
+      </c>
+      <c r="H59" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C59)</f>
+        <v>20</v>
+      </c>
+      <c r="I59" s="0" t="str">
+        <f aca="false">IF(AND($D59&gt;0,$H59=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B60" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A60,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C60" s="13" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D60" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A60,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E60" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C60,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D60)</f>
+        <v>1</v>
+      </c>
+      <c r="F60" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C60,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D60)</f>
+        <v>5</v>
+      </c>
+      <c r="G60" s="0" t="n">
+        <f aca="false">IF($D60=0,0,$E60/$D60)</f>
+        <v>0.166666666666667</v>
+      </c>
+      <c r="H60" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C60)</f>
+        <v>18</v>
+      </c>
+      <c r="I60" s="0" t="str">
+        <f aca="false">IF(AND($D60&gt;0,$H60=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B61" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A61,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C61" s="13" t="s">
+        <v>1848</v>
+      </c>
+      <c r="D61" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A61,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E61" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C61,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D61)</f>
+        <v>1</v>
+      </c>
+      <c r="F61" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C61,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D61)</f>
+        <v>5</v>
+      </c>
+      <c r="G61" s="0" t="n">
+        <f aca="false">IF($D61=0,0,$E61/$D61)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H61" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C61)</f>
+        <v>6</v>
+      </c>
+      <c r="I61" s="0" t="str">
+        <f aca="false">IF(AND($D61&gt;0,$H61=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B62" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A62,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C62" s="13" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D62" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A62,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E62" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C62,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D62)</f>
+        <v>2</v>
+      </c>
+      <c r="F62" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C62,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D62)</f>
+        <v>5</v>
+      </c>
+      <c r="G62" s="0" t="n">
+        <f aca="false">IF($D62=0,0,$E62/$D62)</f>
+        <v>0.285714285714286</v>
+      </c>
+      <c r="H62" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C62)</f>
+        <v>17</v>
+      </c>
+      <c r="I62" s="0" t="str">
+        <f aca="false">IF(AND($D62&gt;0,$H62=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B63" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A63,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C63" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="D63" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A63,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>15</v>
+      </c>
+      <c r="E63" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C63,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D63)</f>
+        <v>6</v>
+      </c>
+      <c r="F63" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C63,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D63)</f>
+        <v>9</v>
+      </c>
+      <c r="G63" s="0" t="n">
+        <f aca="false">IF($D63=0,0,$E63/$D63)</f>
+        <v>0.4</v>
+      </c>
+      <c r="H63" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C63)</f>
+        <v>26</v>
+      </c>
+      <c r="I63" s="0" t="str">
+        <f aca="false">IF(AND($D63&gt;0,$H63=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B64" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A64,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C64" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D64" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A64,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>20</v>
+      </c>
+      <c r="E64" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C64,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D64)</f>
+        <v>10</v>
+      </c>
+      <c r="F64" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C64,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D64)</f>
+        <v>10</v>
+      </c>
+      <c r="G64" s="0" t="n">
+        <f aca="false">IF($D64=0,0,$E64/$D64)</f>
+        <v>0.5</v>
+      </c>
+      <c r="H64" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C64)</f>
+        <v>40</v>
+      </c>
+      <c r="I64" s="0" t="str">
+        <f aca="false">IF(AND($D64&gt;0,$H64=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B65" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A65,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C65" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="D65" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A65,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E65" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C65,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D65)</f>
+        <v>0</v>
+      </c>
+      <c r="F65" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C65,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D65)</f>
+        <v>0</v>
+      </c>
+      <c r="G65" s="0" t="n">
+        <f aca="false">IF($D65=0,0,$E65/$D65)</f>
+        <v>0</v>
+      </c>
+      <c r="H65" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C65)</f>
+        <v>11</v>
+      </c>
+      <c r="I65" s="0" t="str">
+        <f aca="false">IF(AND($D65&gt;0,$H65=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B66" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A66,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C66" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D66" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A66,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E66" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C66,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D66)</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C66,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D66)</f>
+        <v>0</v>
+      </c>
+      <c r="G66" s="0" t="n">
+        <f aca="false">IF($D66=0,0,$E66/$D66)</f>
+        <v>0</v>
+      </c>
+      <c r="H66" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C66)</f>
+        <v>20</v>
+      </c>
+      <c r="I66" s="0" t="str">
+        <f aca="false">IF(AND($D66&gt;0,$H66=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B67" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A67,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C67" s="13" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D67" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A67,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>25</v>
+      </c>
+      <c r="E67" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C67,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D67)</f>
+        <v>4</v>
+      </c>
+      <c r="F67" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C67,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D67)</f>
+        <v>21</v>
+      </c>
+      <c r="G67" s="0" t="n">
+        <f aca="false">IF($D67=0,0,$E67/$D67)</f>
+        <v>0.16</v>
+      </c>
+      <c r="H67" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C67)</f>
+        <v>36</v>
+      </c>
+      <c r="I67" s="0" t="str">
+        <f aca="false">IF(AND($D67&gt;0,$H67=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B68" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A68,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C68" s="13" t="s">
+        <v>1480</v>
+      </c>
+      <c r="D68" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A68,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E68" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C68,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D68)</f>
+        <v>0</v>
+      </c>
+      <c r="F68" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C68,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D68)</f>
+        <v>7</v>
+      </c>
+      <c r="G68" s="0" t="n">
+        <f aca="false">IF($D68=0,0,$E68/$D68)</f>
+        <v>0</v>
+      </c>
+      <c r="H68" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C68)</f>
+        <v>9</v>
+      </c>
+      <c r="I68" s="0" t="str">
+        <f aca="false">IF(AND($D68&gt;0,$H68=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B69" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A69,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C69" s="13" t="s">
+        <v>1847</v>
+      </c>
+      <c r="D69" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A69,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E69" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C69,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D69)</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C69,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D69)</f>
+        <v>7</v>
+      </c>
+      <c r="G69" s="0" t="n">
+        <f aca="false">IF($D69=0,0,$E69/$D69)</f>
+        <v>0</v>
+      </c>
+      <c r="H69" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C69)</f>
+        <v>11</v>
+      </c>
+      <c r="I69" s="0" t="str">
+        <f aca="false">IF(AND($D69&gt;0,$H69=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B70" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A70,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C70" s="13" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D70" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A70,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>11</v>
+      </c>
+      <c r="E70" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C70,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D70)</f>
+        <v>2</v>
+      </c>
+      <c r="F70" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C70,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D70)</f>
+        <v>8</v>
+      </c>
+      <c r="G70" s="0" t="n">
+        <f aca="false">IF($D70=0,0,$E70/$D70)</f>
+        <v>0.181818181818182</v>
+      </c>
+      <c r="H70" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C70)</f>
+        <v>10</v>
+      </c>
+      <c r="I70" s="0" t="str">
+        <f aca="false">IF(AND($D70&gt;0,$H70=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B71" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A71,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C71" s="13" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D71" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A71,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E71" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C71,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D71)</f>
+        <v>2</v>
+      </c>
+      <c r="F71" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C71,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D71)</f>
+        <v>4</v>
+      </c>
+      <c r="G71" s="0" t="n">
+        <f aca="false">IF($D71=0,0,$E71/$D71)</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="H71" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C71)</f>
+        <v>20</v>
+      </c>
+      <c r="I71" s="0" t="str">
+        <f aca="false">IF(AND($D71&gt;0,$H71=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B72" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A72,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C72" s="13" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D72" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A72,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>10</v>
+      </c>
+      <c r="E72" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C72,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D72)</f>
+        <v>5</v>
+      </c>
+      <c r="F72" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C72,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D72)</f>
+        <v>5</v>
+      </c>
+      <c r="G72" s="0" t="n">
+        <f aca="false">IF($D72=0,0,$E72/$D72)</f>
+        <v>0.5</v>
+      </c>
+      <c r="H72" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C72)</f>
+        <v>20</v>
+      </c>
+      <c r="I72" s="0" t="str">
+        <f aca="false">IF(AND($D72&gt;0,$H72=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B73" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A73,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C73" s="13" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D73" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A73,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E73" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C73,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D73)</f>
+        <v>1</v>
+      </c>
+      <c r="F73" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C73,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D73)</f>
+        <v>6</v>
+      </c>
+      <c r="G73" s="0" t="n">
+        <f aca="false">IF($D73=0,0,$E73/$D73)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H73" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C73)</f>
+        <v>18</v>
+      </c>
+      <c r="I73" s="0" t="str">
+        <f aca="false">IF(AND($D73&gt;0,$H73=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B74" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A74,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C74" s="13" t="s">
+        <v>1848</v>
+      </c>
+      <c r="D74" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A74,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>5</v>
+      </c>
+      <c r="E74" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C74,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D74)</f>
+        <v>1</v>
+      </c>
+      <c r="F74" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C74,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D74)</f>
+        <v>4</v>
+      </c>
+      <c r="G74" s="0" t="n">
+        <f aca="false">IF($D74=0,0,$E74/$D74)</f>
+        <v>0.2</v>
+      </c>
+      <c r="H74" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C74)</f>
+        <v>6</v>
+      </c>
+      <c r="I74" s="0" t="str">
+        <f aca="false">IF(AND($D74&gt;0,$H74=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B75" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A75,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C75" s="13" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D75" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A75,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E75" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C75,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D75)</f>
+        <v>2</v>
+      </c>
+      <c r="F75" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C75,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D75)</f>
+        <v>5</v>
+      </c>
+      <c r="G75" s="0" t="n">
+        <f aca="false">IF($D75=0,0,$E75/$D75)</f>
+        <v>0.285714285714286</v>
+      </c>
+      <c r="H75" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C75)</f>
+        <v>17</v>
+      </c>
+      <c r="I75" s="0" t="str">
+        <f aca="false">IF(AND($D75&gt;0,$H75=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B76" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A76,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C76" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="D76" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A76,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>13</v>
+      </c>
+      <c r="E76" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C76,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D76)</f>
+        <v>6</v>
+      </c>
+      <c r="F76" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C76,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D76)</f>
+        <v>7</v>
+      </c>
+      <c r="G76" s="0" t="n">
+        <f aca="false">IF($D76=0,0,$E76/$D76)</f>
+        <v>0.461538461538462</v>
+      </c>
+      <c r="H76" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C76)</f>
+        <v>26</v>
+      </c>
+      <c r="I76" s="0" t="str">
+        <f aca="false">IF(AND($D76&gt;0,$H76=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B77" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A77,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C77" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D77" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A77,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>22</v>
+      </c>
+      <c r="E77" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C77,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D77)</f>
+        <v>11</v>
+      </c>
+      <c r="F77" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C77,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D77)</f>
+        <v>11</v>
+      </c>
+      <c r="G77" s="0" t="n">
+        <f aca="false">IF($D77=0,0,$E77/$D77)</f>
+        <v>0.5</v>
+      </c>
+      <c r="H77" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C77)</f>
+        <v>40</v>
+      </c>
+      <c r="I77" s="0" t="str">
+        <f aca="false">IF(AND($D77&gt;0,$H77=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B78" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A78,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C78" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="D78" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A78,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E78" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C78,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D78)</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C78,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D78)</f>
+        <v>0</v>
+      </c>
+      <c r="G78" s="0" t="n">
+        <f aca="false">IF($D78=0,0,$E78/$D78)</f>
+        <v>0</v>
+      </c>
+      <c r="H78" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C78)</f>
+        <v>11</v>
+      </c>
+      <c r="I78" s="0" t="str">
+        <f aca="false">IF(AND($D78&gt;0,$H78=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="13" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B79" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A79,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C79" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D79" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A79,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E79" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C79,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D79)</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C79,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D79)</f>
+        <v>0</v>
+      </c>
+      <c r="G79" s="0" t="n">
+        <f aca="false">IF($D79=0,0,$E79/$D79)</f>
+        <v>0</v>
+      </c>
+      <c r="H79" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C79)</f>
+        <v>20</v>
+      </c>
+      <c r="I79" s="0" t="str">
+        <f aca="false">IF(AND($D79&gt;0,$H79=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v83: average only Kan, Channel 12 and Channel 13 exit polls
סקר 2026 column B now averages the three main TV exit polls (כאן חדשות,
חדשות 12, חדשות 13) instead of five; Channel 14, i24 and Channel 16 stay
in סקרים לפי ערוץ but no longer feed the average.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C84BdUz8Pbr2phmrWK39vV
</commit_message>
<xml_diff>
--- a/party-comparison-updated-v83.xlsx
+++ b/party-comparison-updated-v83.xlsx
@@ -133,7 +133,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">5 מדגמי הטלוויזיה (27.10.2026) מתוך סקרים לפי ערוץ - ללא ערוץ 16, שפרסם רק מדגם ראשון. מפלגה שאינה במדגמים = 0.</t>
+          <t xml:space="preserve">3 מדגמי הטלוויזיה (27.10.2026) מתוך סקרים לפי ערוץ: כאן חדשות, חדשות 12, חדשות 13. מפלגה שאינה במדגמים = 0.</t>
         </r>
       </text>
     </comment>
@@ -42090,16 +42090,16 @@
         <v>1474</v>
       </c>
       <c r="B2" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A2,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
-        <v>27.8</v>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A2,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
+        <v>27</v>
       </c>
       <c r="C2" s="1" t="n">
         <f aca="false">ROUND(B2,0)</f>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D2" s="1" t="n">
         <f aca="false">IF(C2&lt;=3,0,C2)</f>
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42107,8 +42107,8 @@
         <v>1488</v>
       </c>
       <c r="B3" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A3,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
-        <v>20.8</v>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A3,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
+        <v>21.3333333333333</v>
       </c>
       <c r="C3" s="1" t="n">
         <f aca="false">ROUND(B3,0)</f>
@@ -42124,8 +42124,8 @@
         <v>1489</v>
       </c>
       <c r="B4" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A4,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
-        <v>12.8</v>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A4,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
+        <v>12.6666666666667</v>
       </c>
       <c r="C4" s="1" t="n">
         <f aca="false">ROUND(B4,0)</f>
@@ -42141,7 +42141,7 @@
         <v>1477</v>
       </c>
       <c r="B5" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A5,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A5,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
         <v>9</v>
       </c>
       <c r="C5" s="1" t="n">
@@ -42158,16 +42158,16 @@
         <v>1490</v>
       </c>
       <c r="B6" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A6,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
-        <v>5.4</v>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A6,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
+        <v>7.33333333333333</v>
       </c>
       <c r="C6" s="1" t="n">
         <f aca="false">ROUND(B6,0)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D6" s="1" t="n">
         <f aca="false">IF(C6&lt;=3,0,C6)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42175,16 +42175,16 @@
         <v>1479</v>
       </c>
       <c r="B7" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A7,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
-        <v>7.4</v>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A7,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
+        <v>6.33333333333333</v>
       </c>
       <c r="C7" s="1" t="n">
         <f aca="false">ROUND(B7,0)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" s="1" t="n">
         <f aca="false">IF(C7&lt;=3,0,C7)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42192,8 +42192,8 @@
         <v>1481</v>
       </c>
       <c r="B8" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A8,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
-        <v>6.4</v>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A8,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
+        <v>6</v>
       </c>
       <c r="C8" s="1" t="n">
         <f aca="false">ROUND(B8,0)</f>
@@ -42209,8 +42209,8 @@
         <v>1480</v>
       </c>
       <c r="B9" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A9,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
-        <v>6.4</v>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A9,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
+        <v>6</v>
       </c>
       <c r="C9" s="1" t="n">
         <f aca="false">ROUND(B9,0)</f>
@@ -42226,8 +42226,8 @@
         <v>1491</v>
       </c>
       <c r="B10" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A10,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
-        <v>10.8</v>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A10,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
+        <v>11.3333333333333</v>
       </c>
       <c r="C10" s="1" t="n">
         <f aca="false">ROUND(B10,0)</f>
@@ -42243,8 +42243,8 @@
         <v>1484</v>
       </c>
       <c r="B11" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A11,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
-        <v>6.2</v>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A11,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
+        <v>6</v>
       </c>
       <c r="C11" s="1" t="n">
         <f aca="false">ROUND(B11,0)</f>
@@ -42260,7 +42260,7 @@
         <v>1482</v>
       </c>
       <c r="B12" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A12,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A12,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
         <v>7</v>
       </c>
       <c r="C12" s="1" t="n">
@@ -42277,7 +42277,7 @@
         <v>1492</v>
       </c>
       <c r="B13" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A13,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A13,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
         <v>0</v>
       </c>
       <c r="C13" s="1" t="n">
@@ -42294,7 +42294,7 @@
         <v>1493</v>
       </c>
       <c r="B14" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A14,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A14,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
         <v>0</v>
       </c>
       <c r="C14" s="1" t="n">
@@ -42311,7 +42311,7 @@
         <v>1494</v>
       </c>
       <c r="B15" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A15,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A15,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
         <v>0</v>
       </c>
       <c r="C15" s="1" t="n">
@@ -42328,7 +42328,7 @@
         <v>1495</v>
       </c>
       <c r="B16" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A16,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A16,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
         <v>0</v>
       </c>
       <c r="C16" s="1" t="n">
@@ -42345,7 +42345,7 @@
         <v>1496</v>
       </c>
       <c r="B17" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A17,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A17,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
         <v>0</v>
       </c>
       <c r="C17" s="1" t="n">
@@ -42362,7 +42362,7 @@
         <v>1497</v>
       </c>
       <c r="B18" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A18,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A18,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
         <v>0</v>
       </c>
       <c r="C18" s="1" t="n">
@@ -42379,7 +42379,7 @@
         <v>1498</v>
       </c>
       <c r="B19" s="1" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A19,'סקרים לפי ערוץ'!$E$1:$R$1,0)),'סקרים לפי ערוץ'!$A:$A,"&lt;&gt;ערוץ 16"),0)</f>
+        <f aca="false">IFERROR(SUMPRODUCT(SUMIF('סקרים לפי ערוץ'!$A:$A,{"כאן חדשות","חדשות 12","חדשות 13"},INDEX('סקרים לפי ערוץ'!$E:$R,0,MATCH($A19,'סקרים לפי ערוץ'!$E$1:$R$1,0))))/3,0)</f>
         <v>0</v>
       </c>
       <c r="C19" s="1" t="n">
@@ -46734,7 +46734,7 @@
       </c>
       <c r="B2" s="1" t="n">
         <f aca="false">INDEX('סקר 2026'!$D:$D,MATCH(A2,'סקר 2026'!$A:$A,0))</f>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,A2,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;B2)</f>
@@ -46742,11 +46742,11 @@
       </c>
       <c r="D2" s="1" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,A2,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;B2)</f>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E2" s="1" t="n">
         <f aca="false">IF(B2=0,0,C2/B2)</f>
-        <v>0.142857142857143</v>
+        <v>0.148148148148148</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>1812</v>
@@ -46870,7 +46870,7 @@
       </c>
       <c r="B6" s="1" t="n">
         <f aca="false">INDEX('סקר 2026'!$D:$D,MATCH(A6,'סקר 2026'!$A:$A,0))</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6" s="1" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,A6,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;B6)</f>
@@ -46878,11 +46878,11 @@
       </c>
       <c r="D6" s="1" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,A6,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;B6)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E6" s="1" t="n">
         <f aca="false">IF(B6=0,0,C6/B6)</f>
-        <v>0.4</v>
+        <v>0.285714285714286</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>1816</v>
@@ -46904,7 +46904,7 @@
       </c>
       <c r="B7" s="1" t="n">
         <f aca="false">INDEX('סקר 2026'!$D:$D,MATCH(A7,'סקר 2026'!$A:$A,0))</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="1" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,A7,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;B7)</f>
@@ -46912,7 +46912,7 @@
       </c>
       <c r="D7" s="1" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,A7,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;B7)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" s="1" t="n">
         <f aca="false">IF(B7=0,0,C7/B7)</f>

</xml_diff>

<commit_message>
Add 5-exit-poll average as its own outlet row
סקרים לפי ערוץ gets a 'ממוצע 5 מדגמים' row: the rounded average of the
Channel 12, 13, Kan, 14 and i24 exit polls, so it gets its own charts and
channel tab like any outlet; חישוב לפי ערוץ is rebuilt to include it.
Its seats are stored as values, not formulas, because
update_html_from_xlsx.py reads this tab without cached values. It is
named avg_5_exit_polls in graphs/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C84BdUz8Pbr2phmrWK39vV
</commit_message>
<xml_diff>
--- a/party-comparison-updated-v83.xlsx
+++ b/party-comparison-updated-v83.xlsx
@@ -337,6 +337,74 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
+    <comment ref="A8" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">ממוצע מעוגל של </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">5 מדגמי הטלוויזיה (</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">חדשות </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">12, חדשות 13, כאן חדשות, ערוץ 14, i24 news). </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">ערכים קבועים ולא נוסחה, כי </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">update_html_from_xlsx.py </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">קורא את הגיליון בלי ערכים מחושבים. אם מדגם משתנה - יש לעדכן גם שורה זו</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="B2" authorId="0">
       <text>
         <r>
@@ -502,7 +570,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7554" uniqueCount="1847">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7583" uniqueCount="1858">
   <si>
     <t xml:space="preserve">מפלגה</t>
   </si>
@@ -7301,13 +7369,393 @@
     <t xml:space="preserve">יצחק כ״ץ</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ממוצע </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">מדגמים</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ממוצע</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 12, 13, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">כאן</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 14, i24</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">מנדטים</t>
   </si>
   <si>
-    <t xml:space="preserve">מועמדים ידועים (סה"כ)</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">מועמדים ידועים </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">סה</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">כ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">הערה</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">חדשות </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ש</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ס</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">רע</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">מ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ביחד </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">בנט</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">לפיד</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ישר</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">!</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">המילואימניקים</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">הכלכלית</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">חדשות </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">13</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ערוץ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ערוץ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -7482,7 +7930,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7532,6 +7980,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -47254,7 +47706,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr defaultColWidth="8.53125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -47628,6 +48080,59 @@
         <v>0</v>
       </c>
       <c r="R7" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>1832</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>1845</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="H8" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="I8" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="K8" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="N8" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="O8" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="P8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -47648,2843 +48153,3311 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr defaultColWidth="8.53125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
         <v>1827</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="13" t="s">
         <v>1828</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>1844</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="D1" s="13" t="s">
+        <v>1846</v>
+      </c>
+      <c r="E1" s="13" t="s">
         <v>1472</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="13" t="s">
         <v>1473</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="13" t="s">
         <v>1807</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>1845</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>1846</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B2" s="1" t="str">
+      <c r="H1" s="13" t="s">
+        <v>1847</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B2" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A2,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="13" t="s">
         <v>1474</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A2,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>27</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C2,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D2)</f>
         <v>4</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C2,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D2)</f>
         <v>23</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G2" s="0" t="n">
         <f aca="false">IF($D2=0,0,$E2/$D2)</f>
         <v>0.148148148148148</v>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C2)</f>
         <v>36</v>
       </c>
-      <c r="I2" s="1" t="str">
+      <c r="I2" s="0" t="str">
         <f aca="false">IF(AND($D2&gt;0,$H2=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B3" s="1" t="str">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B3" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A3,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="13" t="s">
         <v>1480</v>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A3,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C3,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D3)</f>
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C3,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D3)</f>
         <v>6</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="G3" s="0" t="n">
         <f aca="false">IF($D3=0,0,$E3/$D3)</f>
         <v>0</v>
       </c>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C3)</f>
         <v>9</v>
       </c>
-      <c r="I3" s="1" t="str">
+      <c r="I3" s="0" t="str">
         <f aca="false">IF(AND($D3&gt;0,$H3=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B4" s="1" t="str">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B4" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A4,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>1479</v>
-      </c>
-      <c r="D4" s="1" t="n">
+      <c r="C4" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D4" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A4,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C4,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D4)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C4,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D4)</f>
         <v>7</v>
       </c>
-      <c r="G4" s="1" t="n">
+      <c r="G4" s="0" t="n">
         <f aca="false">IF($D4=0,0,$E4/$D4)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C4)</f>
         <v>11</v>
       </c>
-      <c r="I4" s="1" t="str">
+      <c r="I4" s="0" t="str">
         <f aca="false">IF(AND($D4&gt;0,$H4=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B5" s="1" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B5" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A5,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="13" t="s">
         <v>1491</v>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A5,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>12</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C5,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D5)</f>
         <v>2</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C5,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D5)</f>
         <v>8</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="G5" s="0" t="n">
         <f aca="false">IF($D5=0,0,$E5/$D5)</f>
         <v>0.166666666666667</v>
       </c>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C5)</f>
         <v>10</v>
       </c>
-      <c r="I5" s="1" t="str">
+      <c r="I5" s="0" t="str">
         <f aca="false">IF(AND($D5&gt;0,$H5=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B6" s="1" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B6" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A6,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="13" t="s">
         <v>1490</v>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A6,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C6,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D6)</f>
         <v>2</v>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C6,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D6)</f>
         <v>5</v>
       </c>
-      <c r="G6" s="1" t="n">
+      <c r="G6" s="0" t="n">
         <f aca="false">IF($D6=0,0,$E6/$D6)</f>
         <v>0.285714285714286</v>
       </c>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C6)</f>
         <v>20</v>
       </c>
-      <c r="I6" s="1" t="str">
+      <c r="I6" s="0" t="str">
         <f aca="false">IF(AND($D6&gt;0,$H6=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B7" s="1" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B7" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A7,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="13" t="s">
         <v>1477</v>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A7,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C7,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D7)</f>
         <v>4</v>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C7,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D7)</f>
         <v>5</v>
       </c>
-      <c r="G7" s="1" t="n">
+      <c r="G7" s="0" t="n">
         <f aca="false">IF($D7=0,0,$E7/$D7)</f>
         <v>0.444444444444444</v>
       </c>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C7)</f>
         <v>20</v>
       </c>
-      <c r="I7" s="1" t="str">
+      <c r="I7" s="0" t="str">
         <f aca="false">IF(AND($D7&gt;0,$H7=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B8" s="1" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B8" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A8,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="13" t="s">
         <v>1484</v>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A8,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C8,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D8)</f>
         <v>1</v>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="F8" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C8,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D8)</f>
         <v>5</v>
       </c>
-      <c r="G8" s="1" t="n">
+      <c r="G8" s="0" t="n">
         <f aca="false">IF($D8=0,0,$E8/$D8)</f>
         <v>0.166666666666667</v>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C8)</f>
         <v>18</v>
       </c>
-      <c r="I8" s="1" t="str">
+      <c r="I8" s="0" t="str">
         <f aca="false">IF(AND($D8&gt;0,$H8=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B9" s="1" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B9" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A9,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>1482</v>
-      </c>
-      <c r="D9" s="1" t="n">
+      <c r="C9" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D9" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A9,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C9,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D9)</f>
         <v>1</v>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="F9" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C9,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D9)</f>
         <v>5</v>
       </c>
-      <c r="G9" s="1" t="n">
+      <c r="G9" s="0" t="n">
         <f aca="false">IF($D9=0,0,$E9/$D9)</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C9)</f>
         <v>6</v>
       </c>
-      <c r="I9" s="1" t="str">
+      <c r="I9" s="0" t="str">
         <f aca="false">IF(AND($D9&gt;0,$H9=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B10" s="1" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B10" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A10,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="13" t="s">
         <v>1481</v>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A10,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C10,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D10)</f>
         <v>2</v>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C10,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D10)</f>
         <v>4</v>
       </c>
-      <c r="G10" s="1" t="n">
+      <c r="G10" s="0" t="n">
         <f aca="false">IF($D10=0,0,$E10/$D10)</f>
         <v>0.333333333333333</v>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C10)</f>
         <v>17</v>
       </c>
-      <c r="I10" s="1" t="str">
+      <c r="I10" s="0" t="str">
         <f aca="false">IF(AND($D10&gt;0,$H10=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B11" s="1" t="str">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B11" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A11,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D11" s="1" t="n">
+      <c r="C11" s="13" t="s">
+        <v>1852</v>
+      </c>
+      <c r="D11" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A11,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>12</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C11,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D11)</f>
         <v>6</v>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="F11" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C11,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D11)</f>
         <v>6</v>
       </c>
-      <c r="G11" s="1" t="n">
+      <c r="G11" s="0" t="n">
         <f aca="false">IF($D11=0,0,$E11/$D11)</f>
         <v>0.5</v>
       </c>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C11)</f>
         <v>26</v>
       </c>
-      <c r="I11" s="1" t="str">
+      <c r="I11" s="0" t="str">
         <f aca="false">IF(AND($D11&gt;0,$H11=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B12" s="1" t="str">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B12" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A12,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>1488</v>
-      </c>
-      <c r="D12" s="1" t="n">
+      <c r="C12" s="13" t="s">
+        <v>1853</v>
+      </c>
+      <c r="D12" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A12,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>21</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C12,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D12)</f>
         <v>11</v>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="F12" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C12,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D12)</f>
         <v>10</v>
       </c>
-      <c r="G12" s="1" t="n">
+      <c r="G12" s="0" t="n">
         <f aca="false">IF($D12=0,0,$E12/$D12)</f>
         <v>0.523809523809524</v>
       </c>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C12)</f>
         <v>40</v>
       </c>
-      <c r="I12" s="1" t="str">
+      <c r="I12" s="0" t="str">
         <f aca="false">IF(AND($D12&gt;0,$H12=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B13" s="1" t="str">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B13" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A13,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="13" t="s">
         <v>1495</v>
       </c>
-      <c r="D13" s="1" t="n">
+      <c r="D13" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A13,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C13,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D13)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C13,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D13)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="1" t="n">
+      <c r="G13" s="0" t="n">
         <f aca="false">IF($D13=0,0,$E13/$D13)</f>
         <v>0</v>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C13)</f>
         <v>11</v>
       </c>
-      <c r="I13" s="1" t="str">
+      <c r="I13" s="0" t="str">
         <f aca="false">IF(AND($D13&gt;0,$H13=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>1831</v>
-      </c>
-      <c r="B14" s="1" t="str">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B14" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A14,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>1496</v>
-      </c>
-      <c r="D14" s="1" t="n">
+      <c r="C14" s="13" t="s">
+        <v>1854</v>
+      </c>
+      <c r="D14" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A14,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C14,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D14)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C14,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D14)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="1" t="n">
+      <c r="G14" s="0" t="n">
         <f aca="false">IF($D14=0,0,$E14/$D14)</f>
         <v>0</v>
       </c>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C14)</f>
         <v>20</v>
       </c>
-      <c r="I14" s="1" t="str">
+      <c r="I14" s="0" t="str">
         <f aca="false">IF(AND($D14&gt;0,$H14=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B15" s="1" t="str">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B15" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A15,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="13" t="s">
         <v>1474</v>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="D15" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A15,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>27</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C15,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D15)</f>
         <v>4</v>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="F15" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C15,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D15)</f>
         <v>23</v>
       </c>
-      <c r="G15" s="1" t="n">
+      <c r="G15" s="0" t="n">
         <f aca="false">IF($D15=0,0,$E15/$D15)</f>
         <v>0.148148148148148</v>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C15)</f>
         <v>36</v>
       </c>
-      <c r="I15" s="1" t="str">
+      <c r="I15" s="0" t="str">
         <f aca="false">IF(AND($D15&gt;0,$H15=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B16" s="1" t="str">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B16" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A16,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="13" t="s">
         <v>1480</v>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A16,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C16,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D16)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="1" t="n">
+      <c r="F16" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C16,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D16)</f>
         <v>6</v>
       </c>
-      <c r="G16" s="1" t="n">
+      <c r="G16" s="0" t="n">
         <f aca="false">IF($D16=0,0,$E16/$D16)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C16)</f>
         <v>9</v>
       </c>
-      <c r="I16" s="1" t="str">
+      <c r="I16" s="0" t="str">
         <f aca="false">IF(AND($D16&gt;0,$H16=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B17" s="1" t="str">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B17" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A17,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>1479</v>
-      </c>
-      <c r="D17" s="1" t="n">
+      <c r="C17" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D17" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A17,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C17,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D17)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="1" t="n">
+      <c r="F17" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C17,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D17)</f>
         <v>6</v>
       </c>
-      <c r="G17" s="1" t="n">
+      <c r="G17" s="0" t="n">
         <f aca="false">IF($D17=0,0,$E17/$D17)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C17)</f>
         <v>11</v>
       </c>
-      <c r="I17" s="1" t="str">
+      <c r="I17" s="0" t="str">
         <f aca="false">IF(AND($D17&gt;0,$H17=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B18" s="1" t="str">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B18" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A18,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="13" t="s">
         <v>1491</v>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A18,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>11</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C18,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D18)</f>
         <v>2</v>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C18,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D18)</f>
         <v>8</v>
       </c>
-      <c r="G18" s="1" t="n">
+      <c r="G18" s="0" t="n">
         <f aca="false">IF($D18=0,0,$E18/$D18)</f>
         <v>0.181818181818182</v>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C18)</f>
         <v>10</v>
       </c>
-      <c r="I18" s="1" t="str">
+      <c r="I18" s="0" t="str">
         <f aca="false">IF(AND($D18&gt;0,$H18=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B19" s="1" t="str">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B19" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A19,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="13" t="s">
         <v>1490</v>
       </c>
-      <c r="D19" s="1" t="n">
+      <c r="D19" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A19,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C19,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D19)</f>
         <v>2</v>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="F19" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C19,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D19)</f>
         <v>5</v>
       </c>
-      <c r="G19" s="1" t="n">
+      <c r="G19" s="0" t="n">
         <f aca="false">IF($D19=0,0,$E19/$D19)</f>
         <v>0.285714285714286</v>
       </c>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C19)</f>
         <v>20</v>
       </c>
-      <c r="I19" s="1" t="str">
+      <c r="I19" s="0" t="str">
         <f aca="false">IF(AND($D19&gt;0,$H19=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B20" s="1" t="str">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B20" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A20,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="13" t="s">
         <v>1477</v>
       </c>
-      <c r="D20" s="1" t="n">
+      <c r="D20" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A20,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C20,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D20)</f>
         <v>4</v>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F20" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C20,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D20)</f>
         <v>5</v>
       </c>
-      <c r="G20" s="1" t="n">
+      <c r="G20" s="0" t="n">
         <f aca="false">IF($D20=0,0,$E20/$D20)</f>
         <v>0.444444444444444</v>
       </c>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C20)</f>
         <v>20</v>
       </c>
-      <c r="I20" s="1" t="str">
+      <c r="I20" s="0" t="str">
         <f aca="false">IF(AND($D20&gt;0,$H20=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B21" s="1" t="str">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B21" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A21,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="13" t="s">
         <v>1484</v>
       </c>
-      <c r="D21" s="1" t="n">
+      <c r="D21" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A21,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C21,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D21)</f>
         <v>1</v>
       </c>
-      <c r="F21" s="1" t="n">
+      <c r="F21" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C21,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D21)</f>
         <v>5</v>
       </c>
-      <c r="G21" s="1" t="n">
+      <c r="G21" s="0" t="n">
         <f aca="false">IF($D21=0,0,$E21/$D21)</f>
         <v>0.166666666666667</v>
       </c>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C21)</f>
         <v>18</v>
       </c>
-      <c r="I21" s="1" t="str">
+      <c r="I21" s="0" t="str">
         <f aca="false">IF(AND($D21&gt;0,$H21=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B22" s="1" t="str">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B22" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A22,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>1482</v>
-      </c>
-      <c r="D22" s="1" t="n">
+      <c r="C22" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D22" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A22,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C22,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D22)</f>
         <v>1</v>
       </c>
-      <c r="F22" s="1" t="n">
+      <c r="F22" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C22,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D22)</f>
         <v>5</v>
       </c>
-      <c r="G22" s="1" t="n">
+      <c r="G22" s="0" t="n">
         <f aca="false">IF($D22=0,0,$E22/$D22)</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C22)</f>
         <v>6</v>
       </c>
-      <c r="I22" s="1" t="str">
+      <c r="I22" s="0" t="str">
         <f aca="false">IF(AND($D22&gt;0,$H22=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B23" s="1" t="str">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B23" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A23,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="13" t="s">
         <v>1481</v>
       </c>
-      <c r="D23" s="1" t="n">
+      <c r="D23" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A23,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C23,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D23)</f>
         <v>2</v>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="F23" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C23,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D23)</f>
         <v>4</v>
       </c>
-      <c r="G23" s="1" t="n">
+      <c r="G23" s="0" t="n">
         <f aca="false">IF($D23=0,0,$E23/$D23)</f>
         <v>0.333333333333333</v>
       </c>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C23)</f>
         <v>17</v>
       </c>
-      <c r="I23" s="1" t="str">
+      <c r="I23" s="0" t="str">
         <f aca="false">IF(AND($D23&gt;0,$H23=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B24" s="1" t="str">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B24" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A24,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D24" s="1" t="n">
+      <c r="C24" s="13" t="s">
+        <v>1852</v>
+      </c>
+      <c r="D24" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A24,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>13</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C24,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D24)</f>
         <v>6</v>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="F24" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C24,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D24)</f>
         <v>7</v>
       </c>
-      <c r="G24" s="1" t="n">
+      <c r="G24" s="0" t="n">
         <f aca="false">IF($D24=0,0,$E24/$D24)</f>
         <v>0.461538461538462</v>
       </c>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C24)</f>
         <v>26</v>
       </c>
-      <c r="I24" s="1" t="str">
+      <c r="I24" s="0" t="str">
         <f aca="false">IF(AND($D24&gt;0,$H24=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B25" s="1" t="str">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B25" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A25,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>1488</v>
-      </c>
-      <c r="D25" s="1" t="n">
+      <c r="C25" s="13" t="s">
+        <v>1853</v>
+      </c>
+      <c r="D25" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A25,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>22</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C25,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D25)</f>
         <v>11</v>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="F25" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C25,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D25)</f>
         <v>11</v>
       </c>
-      <c r="G25" s="1" t="n">
+      <c r="G25" s="0" t="n">
         <f aca="false">IF($D25=0,0,$E25/$D25)</f>
         <v>0.5</v>
       </c>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C25)</f>
         <v>40</v>
       </c>
-      <c r="I25" s="1" t="str">
+      <c r="I25" s="0" t="str">
         <f aca="false">IF(AND($D25&gt;0,$H25=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B26" s="1" t="str">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B26" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A26,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="13" t="s">
         <v>1495</v>
       </c>
-      <c r="D26" s="1" t="n">
+      <c r="D26" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A26,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C26,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D26)</f>
         <v>0</v>
       </c>
-      <c r="F26" s="1" t="n">
+      <c r="F26" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C26,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D26)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="1" t="n">
+      <c r="G26" s="0" t="n">
         <f aca="false">IF($D26=0,0,$E26/$D26)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C26)</f>
         <v>11</v>
       </c>
-      <c r="I26" s="1" t="str">
+      <c r="I26" s="0" t="str">
         <f aca="false">IF(AND($D26&gt;0,$H26=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>1834</v>
-      </c>
-      <c r="B27" s="1" t="str">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B27" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A27,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>1496</v>
-      </c>
-      <c r="D27" s="1" t="n">
+      <c r="C27" s="13" t="s">
+        <v>1854</v>
+      </c>
+      <c r="D27" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A27,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C27,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D27)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="1" t="n">
+      <c r="F27" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C27,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D27)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="1" t="n">
+      <c r="G27" s="0" t="n">
         <f aca="false">IF($D27=0,0,$E27/$D27)</f>
         <v>0</v>
       </c>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C27)</f>
         <v>20</v>
       </c>
-      <c r="I27" s="1" t="str">
+      <c r="I27" s="0" t="str">
         <f aca="false">IF(AND($D27&gt;0,$H27=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B28" s="1" t="str">
+      <c r="B28" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A28,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="13" t="s">
         <v>1474</v>
       </c>
-      <c r="D28" s="1" t="n">
+      <c r="D28" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A28,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>27</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C28,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D28)</f>
         <v>4</v>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="F28" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C28,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D28)</f>
         <v>23</v>
       </c>
-      <c r="G28" s="1" t="n">
+      <c r="G28" s="0" t="n">
         <f aca="false">IF($D28=0,0,$E28/$D28)</f>
         <v>0.148148148148148</v>
       </c>
-      <c r="H28" s="1" t="n">
+      <c r="H28" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C28)</f>
         <v>36</v>
       </c>
-      <c r="I28" s="1" t="str">
+      <c r="I28" s="0" t="str">
         <f aca="false">IF(AND($D28&gt;0,$H28=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B29" s="1" t="str">
+      <c r="B29" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A29,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="13" t="s">
         <v>1480</v>
       </c>
-      <c r="D29" s="1" t="n">
+      <c r="D29" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A29,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E29" s="1" t="n">
+      <c r="E29" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C29,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D29)</f>
         <v>0</v>
       </c>
-      <c r="F29" s="1" t="n">
+      <c r="F29" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C29,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D29)</f>
         <v>6</v>
       </c>
-      <c r="G29" s="1" t="n">
+      <c r="G29" s="0" t="n">
         <f aca="false">IF($D29=0,0,$E29/$D29)</f>
         <v>0</v>
       </c>
-      <c r="H29" s="1" t="n">
+      <c r="H29" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C29)</f>
         <v>9</v>
       </c>
-      <c r="I29" s="1" t="str">
+      <c r="I29" s="0" t="str">
         <f aca="false">IF(AND($D29&gt;0,$H29=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B30" s="1" t="str">
+      <c r="B30" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A30,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>1479</v>
-      </c>
-      <c r="D30" s="1" t="n">
+      <c r="C30" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D30" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A30,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="E30" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C30,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D30)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="1" t="n">
+      <c r="F30" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C30,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D30)</f>
         <v>6</v>
       </c>
-      <c r="G30" s="1" t="n">
+      <c r="G30" s="0" t="n">
         <f aca="false">IF($D30=0,0,$E30/$D30)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C30)</f>
         <v>11</v>
       </c>
-      <c r="I30" s="1" t="str">
+      <c r="I30" s="0" t="str">
         <f aca="false">IF(AND($D30&gt;0,$H30=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B31" s="1" t="str">
+      <c r="B31" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A31,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="13" t="s">
         <v>1491</v>
       </c>
-      <c r="D31" s="1" t="n">
+      <c r="D31" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A31,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>11</v>
       </c>
-      <c r="E31" s="1" t="n">
+      <c r="E31" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C31,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D31)</f>
         <v>2</v>
       </c>
-      <c r="F31" s="1" t="n">
+      <c r="F31" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C31,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D31)</f>
         <v>8</v>
       </c>
-      <c r="G31" s="1" t="n">
+      <c r="G31" s="0" t="n">
         <f aca="false">IF($D31=0,0,$E31/$D31)</f>
         <v>0.181818181818182</v>
       </c>
-      <c r="H31" s="1" t="n">
+      <c r="H31" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C31)</f>
         <v>10</v>
       </c>
-      <c r="I31" s="1" t="str">
+      <c r="I31" s="0" t="str">
         <f aca="false">IF(AND($D31&gt;0,$H31=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B32" s="1" t="str">
+      <c r="B32" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A32,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="13" t="s">
         <v>1490</v>
       </c>
-      <c r="D32" s="1" t="n">
+      <c r="D32" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A32,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="E32" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C32,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D32)</f>
         <v>2</v>
       </c>
-      <c r="F32" s="1" t="n">
+      <c r="F32" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C32,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D32)</f>
         <v>6</v>
       </c>
-      <c r="G32" s="1" t="n">
+      <c r="G32" s="0" t="n">
         <f aca="false">IF($D32=0,0,$E32/$D32)</f>
         <v>0.25</v>
       </c>
-      <c r="H32" s="1" t="n">
+      <c r="H32" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C32)</f>
         <v>20</v>
       </c>
-      <c r="I32" s="1" t="str">
+      <c r="I32" s="0" t="str">
         <f aca="false">IF(AND($D32&gt;0,$H32=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B33" s="1" t="str">
+      <c r="B33" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A33,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="13" t="s">
         <v>1477</v>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D33" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A33,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
-      <c r="E33" s="1" t="n">
+      <c r="E33" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C33,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D33)</f>
         <v>4</v>
       </c>
-      <c r="F33" s="1" t="n">
+      <c r="F33" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C33,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D33)</f>
         <v>5</v>
       </c>
-      <c r="G33" s="1" t="n">
+      <c r="G33" s="0" t="n">
         <f aca="false">IF($D33=0,0,$E33/$D33)</f>
         <v>0.444444444444444</v>
       </c>
-      <c r="H33" s="1" t="n">
+      <c r="H33" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C33)</f>
         <v>20</v>
       </c>
-      <c r="I33" s="1" t="str">
+      <c r="I33" s="0" t="str">
         <f aca="false">IF(AND($D33&gt;0,$H33=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B34" s="1" t="str">
+      <c r="B34" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A34,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="13" t="s">
         <v>1484</v>
       </c>
-      <c r="D34" s="1" t="n">
+      <c r="D34" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A34,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E34" s="1" t="n">
+      <c r="E34" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C34,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D34)</f>
         <v>1</v>
       </c>
-      <c r="F34" s="1" t="n">
+      <c r="F34" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C34,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D34)</f>
         <v>5</v>
       </c>
-      <c r="G34" s="1" t="n">
+      <c r="G34" s="0" t="n">
         <f aca="false">IF($D34=0,0,$E34/$D34)</f>
         <v>0.166666666666667</v>
       </c>
-      <c r="H34" s="1" t="n">
+      <c r="H34" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C34)</f>
         <v>18</v>
       </c>
-      <c r="I34" s="1" t="str">
+      <c r="I34" s="0" t="str">
         <f aca="false">IF(AND($D34&gt;0,$H34=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B35" s="1" t="str">
+      <c r="B35" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A35,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C35" s="3" t="s">
-        <v>1482</v>
-      </c>
-      <c r="D35" s="1" t="n">
+      <c r="C35" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D35" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A35,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E35" s="1" t="n">
+      <c r="E35" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C35,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D35)</f>
         <v>1</v>
       </c>
-      <c r="F35" s="1" t="n">
+      <c r="F35" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C35,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D35)</f>
         <v>5</v>
       </c>
-      <c r="G35" s="1" t="n">
+      <c r="G35" s="0" t="n">
         <f aca="false">IF($D35=0,0,$E35/$D35)</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="H35" s="1" t="n">
+      <c r="H35" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C35)</f>
         <v>6</v>
       </c>
-      <c r="I35" s="1" t="str">
+      <c r="I35" s="0" t="str">
         <f aca="false">IF(AND($D35&gt;0,$H35=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B36" s="1" t="str">
+      <c r="B36" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A36,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="13" t="s">
         <v>1481</v>
       </c>
-      <c r="D36" s="1" t="n">
+      <c r="D36" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A36,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E36" s="1" t="n">
+      <c r="E36" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C36,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D36)</f>
         <v>2</v>
       </c>
-      <c r="F36" s="1" t="n">
+      <c r="F36" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C36,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D36)</f>
         <v>4</v>
       </c>
-      <c r="G36" s="1" t="n">
+      <c r="G36" s="0" t="n">
         <f aca="false">IF($D36=0,0,$E36/$D36)</f>
         <v>0.333333333333333</v>
       </c>
-      <c r="H36" s="1" t="n">
+      <c r="H36" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C36)</f>
         <v>17</v>
       </c>
-      <c r="I36" s="1" t="str">
+      <c r="I36" s="0" t="str">
         <f aca="false">IF(AND($D36&gt;0,$H36=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B37" s="1" t="str">
+      <c r="B37" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A37,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C37" s="3" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D37" s="1" t="n">
+      <c r="C37" s="13" t="s">
+        <v>1852</v>
+      </c>
+      <c r="D37" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A37,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>13</v>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C37,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D37)</f>
         <v>6</v>
       </c>
-      <c r="F37" s="1" t="n">
+      <c r="F37" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C37,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D37)</f>
         <v>7</v>
       </c>
-      <c r="G37" s="1" t="n">
+      <c r="G37" s="0" t="n">
         <f aca="false">IF($D37=0,0,$E37/$D37)</f>
         <v>0.461538461538462</v>
       </c>
-      <c r="H37" s="1" t="n">
+      <c r="H37" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C37)</f>
         <v>26</v>
       </c>
-      <c r="I37" s="1" t="str">
+      <c r="I37" s="0" t="str">
         <f aca="false">IF(AND($D37&gt;0,$H37=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B38" s="1" t="str">
+      <c r="B38" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A38,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C38" s="3" t="s">
-        <v>1488</v>
-      </c>
-      <c r="D38" s="1" t="n">
+      <c r="C38" s="13" t="s">
+        <v>1853</v>
+      </c>
+      <c r="D38" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A38,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>21</v>
       </c>
-      <c r="E38" s="1" t="n">
+      <c r="E38" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C38,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D38)</f>
         <v>11</v>
       </c>
-      <c r="F38" s="1" t="n">
+      <c r="F38" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C38,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D38)</f>
         <v>10</v>
       </c>
-      <c r="G38" s="1" t="n">
+      <c r="G38" s="0" t="n">
         <f aca="false">IF($D38=0,0,$E38/$D38)</f>
         <v>0.523809523809524</v>
       </c>
-      <c r="H38" s="1" t="n">
+      <c r="H38" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C38)</f>
         <v>40</v>
       </c>
-      <c r="I38" s="1" t="str">
+      <c r="I38" s="0" t="str">
         <f aca="false">IF(AND($D38&gt;0,$H38=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B39" s="1" t="str">
+      <c r="B39" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A39,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="13" t="s">
         <v>1495</v>
       </c>
-      <c r="D39" s="1" t="n">
+      <c r="D39" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A39,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E39" s="1" t="n">
+      <c r="E39" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C39,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D39)</f>
         <v>0</v>
       </c>
-      <c r="F39" s="1" t="n">
+      <c r="F39" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C39,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D39)</f>
         <v>0</v>
       </c>
-      <c r="G39" s="1" t="n">
+      <c r="G39" s="0" t="n">
         <f aca="false">IF($D39=0,0,$E39/$D39)</f>
         <v>0</v>
       </c>
-      <c r="H39" s="1" t="n">
+      <c r="H39" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C39)</f>
         <v>11</v>
       </c>
-      <c r="I39" s="1" t="str">
+      <c r="I39" s="0" t="str">
         <f aca="false">IF(AND($D39&gt;0,$H39=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13" t="s">
         <v>1836</v>
       </c>
-      <c r="B40" s="1" t="str">
+      <c r="B40" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A40,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>1496</v>
-      </c>
-      <c r="D40" s="1" t="n">
+      <c r="C40" s="13" t="s">
+        <v>1854</v>
+      </c>
+      <c r="D40" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A40,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E40" s="1" t="n">
+      <c r="E40" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C40,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D40)</f>
         <v>0</v>
       </c>
-      <c r="F40" s="1" t="n">
+      <c r="F40" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C40,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D40)</f>
         <v>0</v>
       </c>
-      <c r="G40" s="1" t="n">
+      <c r="G40" s="0" t="n">
         <f aca="false">IF($D40=0,0,$E40/$D40)</f>
         <v>0</v>
       </c>
-      <c r="H40" s="1" t="n">
+      <c r="H40" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C40)</f>
         <v>20</v>
       </c>
-      <c r="I40" s="1" t="str">
+      <c r="I40" s="0" t="str">
         <f aca="false">IF(AND($D40&gt;0,$H40=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B41" s="1" t="str">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B41" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A41,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="13" t="s">
         <v>1474</v>
       </c>
-      <c r="D41" s="1" t="n">
+      <c r="D41" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A41,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>31</v>
       </c>
-      <c r="E41" s="1" t="n">
+      <c r="E41" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C41,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D41)</f>
         <v>4</v>
       </c>
-      <c r="F41" s="1" t="n">
+      <c r="F41" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C41,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D41)</f>
         <v>27</v>
       </c>
-      <c r="G41" s="1" t="n">
+      <c r="G41" s="0" t="n">
         <f aca="false">IF($D41=0,0,$E41/$D41)</f>
         <v>0.129032258064516</v>
       </c>
-      <c r="H41" s="1" t="n">
+      <c r="H41" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C41)</f>
         <v>36</v>
       </c>
-      <c r="I41" s="1" t="str">
+      <c r="I41" s="0" t="str">
         <f aca="false">IF(AND($D41&gt;0,$H41=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B42" s="1" t="str">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B42" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A42,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="13" t="s">
         <v>1480</v>
       </c>
-      <c r="D42" s="1" t="n">
+      <c r="D42" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A42,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E42" s="1" t="n">
+      <c r="E42" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C42,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D42)</f>
         <v>0</v>
       </c>
-      <c r="F42" s="1" t="n">
+      <c r="F42" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C42,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D42)</f>
         <v>7</v>
       </c>
-      <c r="G42" s="1" t="n">
+      <c r="G42" s="0" t="n">
         <f aca="false">IF($D42=0,0,$E42/$D42)</f>
         <v>0</v>
       </c>
-      <c r="H42" s="1" t="n">
+      <c r="H42" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C42)</f>
         <v>9</v>
       </c>
-      <c r="I42" s="1" t="str">
+      <c r="I42" s="0" t="str">
         <f aca="false">IF(AND($D42&gt;0,$H42=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B43" s="1" t="str">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B43" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A43,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C43" s="3" t="s">
-        <v>1479</v>
-      </c>
-      <c r="D43" s="1" t="n">
+      <c r="C43" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D43" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A43,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>10</v>
       </c>
-      <c r="E43" s="1" t="n">
+      <c r="E43" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C43,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D43)</f>
         <v>0</v>
       </c>
-      <c r="F43" s="1" t="n">
+      <c r="F43" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C43,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D43)</f>
         <v>10</v>
       </c>
-      <c r="G43" s="1" t="n">
+      <c r="G43" s="0" t="n">
         <f aca="false">IF($D43=0,0,$E43/$D43)</f>
         <v>0</v>
       </c>
-      <c r="H43" s="1" t="n">
+      <c r="H43" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C43)</f>
         <v>11</v>
       </c>
-      <c r="I43" s="1" t="str">
+      <c r="I43" s="0" t="str">
         <f aca="false">IF(AND($D43&gt;0,$H43=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B44" s="1" t="str">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B44" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A44,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="13" t="s">
         <v>1491</v>
       </c>
-      <c r="D44" s="1" t="n">
+      <c r="D44" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A44,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>11</v>
       </c>
-      <c r="E44" s="1" t="n">
+      <c r="E44" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C44,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D44)</f>
         <v>2</v>
       </c>
-      <c r="F44" s="1" t="n">
+      <c r="F44" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C44,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D44)</f>
         <v>8</v>
       </c>
-      <c r="G44" s="1" t="n">
+      <c r="G44" s="0" t="n">
         <f aca="false">IF($D44=0,0,$E44/$D44)</f>
         <v>0.181818181818182</v>
       </c>
-      <c r="H44" s="1" t="n">
+      <c r="H44" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C44)</f>
         <v>10</v>
       </c>
-      <c r="I44" s="1" t="str">
+      <c r="I44" s="0" t="str">
         <f aca="false">IF(AND($D44&gt;0,$H44=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B45" s="1" t="str">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B45" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A45,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="13" t="s">
         <v>1490</v>
       </c>
-      <c r="D45" s="1" t="n">
+      <c r="D45" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A45,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E45" s="1" t="n">
+      <c r="E45" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C45,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D45)</f>
         <v>0</v>
       </c>
-      <c r="F45" s="1" t="n">
+      <c r="F45" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C45,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D45)</f>
         <v>0</v>
       </c>
-      <c r="G45" s="1" t="n">
+      <c r="G45" s="0" t="n">
         <f aca="false">IF($D45=0,0,$E45/$D45)</f>
         <v>0</v>
       </c>
-      <c r="H45" s="1" t="n">
+      <c r="H45" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C45)</f>
         <v>20</v>
       </c>
-      <c r="I45" s="1" t="str">
+      <c r="I45" s="0" t="str">
         <f aca="false">IF(AND($D45&gt;0,$H45=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B46" s="1" t="str">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B46" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A46,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="13" t="s">
         <v>1477</v>
       </c>
-      <c r="D46" s="1" t="n">
+      <c r="D46" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A46,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
-      <c r="E46" s="1" t="n">
+      <c r="E46" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C46,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D46)</f>
         <v>4</v>
       </c>
-      <c r="F46" s="1" t="n">
+      <c r="F46" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C46,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D46)</f>
         <v>5</v>
       </c>
-      <c r="G46" s="1" t="n">
+      <c r="G46" s="0" t="n">
         <f aca="false">IF($D46=0,0,$E46/$D46)</f>
         <v>0.444444444444444</v>
       </c>
-      <c r="H46" s="1" t="n">
+      <c r="H46" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C46)</f>
         <v>20</v>
       </c>
-      <c r="I46" s="1" t="str">
+      <c r="I46" s="0" t="str">
         <f aca="false">IF(AND($D46&gt;0,$H46=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B47" s="1" t="str">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B47" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A47,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="13" t="s">
         <v>1484</v>
       </c>
-      <c r="D47" s="1" t="n">
+      <c r="D47" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A47,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E47" s="1" t="n">
+      <c r="E47" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C47,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D47)</f>
         <v>1</v>
       </c>
-      <c r="F47" s="1" t="n">
+      <c r="F47" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C47,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D47)</f>
         <v>6</v>
       </c>
-      <c r="G47" s="1" t="n">
+      <c r="G47" s="0" t="n">
         <f aca="false">IF($D47=0,0,$E47/$D47)</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="H47" s="1" t="n">
+      <c r="H47" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C47)</f>
         <v>18</v>
       </c>
-      <c r="I47" s="1" t="str">
+      <c r="I47" s="0" t="str">
         <f aca="false">IF(AND($D47&gt;0,$H47=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B48" s="1" t="str">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B48" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A48,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C48" s="3" t="s">
-        <v>1482</v>
-      </c>
-      <c r="D48" s="1" t="n">
+      <c r="C48" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D48" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A48,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E48" s="1" t="n">
+      <c r="E48" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C48,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D48)</f>
         <v>1</v>
       </c>
-      <c r="F48" s="1" t="n">
+      <c r="F48" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C48,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D48)</f>
         <v>5</v>
       </c>
-      <c r="G48" s="1" t="n">
+      <c r="G48" s="0" t="n">
         <f aca="false">IF($D48=0,0,$E48/$D48)</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="H48" s="1" t="n">
+      <c r="H48" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C48)</f>
         <v>6</v>
       </c>
-      <c r="I48" s="1" t="str">
+      <c r="I48" s="0" t="str">
         <f aca="false">IF(AND($D48&gt;0,$H48=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B49" s="1" t="str">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B49" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A49,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C49" s="13" t="s">
         <v>1481</v>
       </c>
-      <c r="D49" s="1" t="n">
+      <c r="D49" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A49,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E49" s="1" t="n">
+      <c r="E49" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C49,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D49)</f>
         <v>2</v>
       </c>
-      <c r="F49" s="1" t="n">
+      <c r="F49" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C49,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D49)</f>
         <v>5</v>
       </c>
-      <c r="G49" s="1" t="n">
+      <c r="G49" s="0" t="n">
         <f aca="false">IF($D49=0,0,$E49/$D49)</f>
         <v>0.285714285714286</v>
       </c>
-      <c r="H49" s="1" t="n">
+      <c r="H49" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C49)</f>
         <v>17</v>
       </c>
-      <c r="I49" s="1" t="str">
+      <c r="I49" s="0" t="str">
         <f aca="false">IF(AND($D49&gt;0,$H49=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B50" s="1" t="str">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B50" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A50,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C50" s="3" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D50" s="1" t="n">
+      <c r="C50" s="13" t="s">
+        <v>1852</v>
+      </c>
+      <c r="D50" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A50,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>11</v>
       </c>
-      <c r="E50" s="1" t="n">
+      <c r="E50" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C50,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D50)</f>
         <v>6</v>
       </c>
-      <c r="F50" s="1" t="n">
+      <c r="F50" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C50,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D50)</f>
         <v>5</v>
       </c>
-      <c r="G50" s="1" t="n">
+      <c r="G50" s="0" t="n">
         <f aca="false">IF($D50=0,0,$E50/$D50)</f>
         <v>0.545454545454545</v>
       </c>
-      <c r="H50" s="1" t="n">
+      <c r="H50" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C50)</f>
         <v>26</v>
       </c>
-      <c r="I50" s="1" t="str">
+      <c r="I50" s="0" t="str">
         <f aca="false">IF(AND($D50&gt;0,$H50=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B51" s="1" t="str">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B51" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A51,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C51" s="3" t="s">
-        <v>1488</v>
-      </c>
-      <c r="D51" s="1" t="n">
+      <c r="C51" s="13" t="s">
+        <v>1853</v>
+      </c>
+      <c r="D51" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A51,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>20</v>
       </c>
-      <c r="E51" s="1" t="n">
+      <c r="E51" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C51,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D51)</f>
         <v>10</v>
       </c>
-      <c r="F51" s="1" t="n">
+      <c r="F51" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C51,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D51)</f>
         <v>10</v>
       </c>
-      <c r="G51" s="1" t="n">
+      <c r="G51" s="0" t="n">
         <f aca="false">IF($D51=0,0,$E51/$D51)</f>
         <v>0.5</v>
       </c>
-      <c r="H51" s="1" t="n">
+      <c r="H51" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C51)</f>
         <v>40</v>
       </c>
-      <c r="I51" s="1" t="str">
+      <c r="I51" s="0" t="str">
         <f aca="false">IF(AND($D51&gt;0,$H51=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B52" s="1" t="str">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B52" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A52,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="13" t="s">
         <v>1495</v>
       </c>
-      <c r="D52" s="1" t="n">
+      <c r="D52" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A52,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E52" s="1" t="n">
+      <c r="E52" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C52,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D52)</f>
         <v>0</v>
       </c>
-      <c r="F52" s="1" t="n">
+      <c r="F52" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C52,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D52)</f>
         <v>0</v>
       </c>
-      <c r="G52" s="1" t="n">
+      <c r="G52" s="0" t="n">
         <f aca="false">IF($D52=0,0,$E52/$D52)</f>
         <v>0</v>
       </c>
-      <c r="H52" s="1" t="n">
+      <c r="H52" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C52)</f>
         <v>11</v>
       </c>
-      <c r="I52" s="1" t="str">
+      <c r="I52" s="0" t="str">
         <f aca="false">IF(AND($D52&gt;0,$H52=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
-        <v>1838</v>
-      </c>
-      <c r="B53" s="1" t="str">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="13" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B53" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A53,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C53" s="3" t="s">
-        <v>1496</v>
-      </c>
-      <c r="D53" s="1" t="n">
+      <c r="C53" s="13" t="s">
+        <v>1854</v>
+      </c>
+      <c r="D53" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A53,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E53" s="1" t="n">
+      <c r="E53" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C53,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D53)</f>
         <v>0</v>
       </c>
-      <c r="F53" s="1" t="n">
+      <c r="F53" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C53,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D53)</f>
         <v>0</v>
       </c>
-      <c r="G53" s="1" t="n">
+      <c r="G53" s="0" t="n">
         <f aca="false">IF($D53=0,0,$E53/$D53)</f>
         <v>0</v>
       </c>
-      <c r="H53" s="1" t="n">
+      <c r="H53" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C53)</f>
         <v>20</v>
       </c>
-      <c r="I53" s="1" t="str">
+      <c r="I53" s="0" t="str">
         <f aca="false">IF(AND($D53&gt;0,$H53=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="1" t="s">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B54" s="1" t="str">
+      <c r="B54" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A54,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="13" t="s">
         <v>1474</v>
       </c>
-      <c r="D54" s="1" t="n">
+      <c r="D54" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A54,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>27</v>
       </c>
-      <c r="E54" s="1" t="n">
+      <c r="E54" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C54,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D54)</f>
         <v>4</v>
       </c>
-      <c r="F54" s="1" t="n">
+      <c r="F54" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C54,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D54)</f>
         <v>23</v>
       </c>
-      <c r="G54" s="1" t="n">
+      <c r="G54" s="0" t="n">
         <f aca="false">IF($D54=0,0,$E54/$D54)</f>
         <v>0.148148148148148</v>
       </c>
-      <c r="H54" s="1" t="n">
+      <c r="H54" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C54)</f>
         <v>36</v>
       </c>
-      <c r="I54" s="1" t="str">
+      <c r="I54" s="0" t="str">
         <f aca="false">IF(AND($D54&gt;0,$H54=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="1" t="s">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B55" s="1" t="str">
+      <c r="B55" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A55,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="13" t="s">
         <v>1480</v>
       </c>
-      <c r="D55" s="1" t="n">
+      <c r="D55" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A55,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E55" s="1" t="n">
+      <c r="E55" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C55,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D55)</f>
         <v>0</v>
       </c>
-      <c r="F55" s="1" t="n">
+      <c r="F55" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C55,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D55)</f>
         <v>7</v>
       </c>
-      <c r="G55" s="1" t="n">
+      <c r="G55" s="0" t="n">
         <f aca="false">IF($D55=0,0,$E55/$D55)</f>
         <v>0</v>
       </c>
-      <c r="H55" s="1" t="n">
+      <c r="H55" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C55)</f>
         <v>9</v>
       </c>
-      <c r="I55" s="1" t="str">
+      <c r="I55" s="0" t="str">
         <f aca="false">IF(AND($D55&gt;0,$H55=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1" t="s">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B56" s="1" t="str">
+      <c r="B56" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A56,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C56" s="3" t="s">
-        <v>1479</v>
-      </c>
-      <c r="D56" s="1" t="n">
+      <c r="C56" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D56" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A56,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>8</v>
       </c>
-      <c r="E56" s="1" t="n">
+      <c r="E56" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C56,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D56)</f>
         <v>0</v>
       </c>
-      <c r="F56" s="1" t="n">
+      <c r="F56" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C56,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D56)</f>
         <v>8</v>
       </c>
-      <c r="G56" s="1" t="n">
+      <c r="G56" s="0" t="n">
         <f aca="false">IF($D56=0,0,$E56/$D56)</f>
         <v>0</v>
       </c>
-      <c r="H56" s="1" t="n">
+      <c r="H56" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C56)</f>
         <v>11</v>
       </c>
-      <c r="I56" s="1" t="str">
+      <c r="I56" s="0" t="str">
         <f aca="false">IF(AND($D56&gt;0,$H56=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="1" t="s">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B57" s="1" t="str">
+      <c r="B57" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A57,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C57" s="13" t="s">
         <v>1491</v>
       </c>
-      <c r="D57" s="1" t="n">
+      <c r="D57" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A57,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
-      <c r="E57" s="1" t="n">
+      <c r="E57" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C57,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D57)</f>
         <v>2</v>
       </c>
-      <c r="F57" s="1" t="n">
+      <c r="F57" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C57,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D57)</f>
         <v>7</v>
       </c>
-      <c r="G57" s="1" t="n">
+      <c r="G57" s="0" t="n">
         <f aca="false">IF($D57=0,0,$E57/$D57)</f>
         <v>0.222222222222222</v>
       </c>
-      <c r="H57" s="1" t="n">
+      <c r="H57" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C57)</f>
         <v>10</v>
       </c>
-      <c r="I57" s="1" t="str">
+      <c r="I57" s="0" t="str">
         <f aca="false">IF(AND($D57&gt;0,$H57=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1" t="s">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B58" s="1" t="str">
+      <c r="B58" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A58,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C58" s="13" t="s">
         <v>1490</v>
       </c>
-      <c r="D58" s="1" t="n">
+      <c r="D58" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A58,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
-      <c r="E58" s="1" t="n">
+      <c r="E58" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C58,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D58)</f>
         <v>2</v>
       </c>
-      <c r="F58" s="1" t="n">
+      <c r="F58" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C58,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D58)</f>
         <v>3</v>
       </c>
-      <c r="G58" s="1" t="n">
+      <c r="G58" s="0" t="n">
         <f aca="false">IF($D58=0,0,$E58/$D58)</f>
         <v>0.4</v>
       </c>
-      <c r="H58" s="1" t="n">
+      <c r="H58" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C58)</f>
         <v>20</v>
       </c>
-      <c r="I58" s="1" t="str">
+      <c r="I58" s="0" t="str">
         <f aca="false">IF(AND($D58&gt;0,$H58=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1" t="s">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B59" s="1" t="str">
+      <c r="B59" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A59,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C59" s="3" t="s">
+      <c r="C59" s="13" t="s">
         <v>1477</v>
       </c>
-      <c r="D59" s="1" t="n">
+      <c r="D59" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A59,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>9</v>
       </c>
-      <c r="E59" s="1" t="n">
+      <c r="E59" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C59,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D59)</f>
         <v>4</v>
       </c>
-      <c r="F59" s="1" t="n">
+      <c r="F59" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C59,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D59)</f>
         <v>5</v>
       </c>
-      <c r="G59" s="1" t="n">
+      <c r="G59" s="0" t="n">
         <f aca="false">IF($D59=0,0,$E59/$D59)</f>
         <v>0.444444444444444</v>
       </c>
-      <c r="H59" s="1" t="n">
+      <c r="H59" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C59)</f>
         <v>20</v>
       </c>
-      <c r="I59" s="1" t="str">
+      <c r="I59" s="0" t="str">
         <f aca="false">IF(AND($D59&gt;0,$H59=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="1" t="s">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B60" s="1" t="str">
+      <c r="B60" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A60,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C60" s="3" t="s">
+      <c r="C60" s="13" t="s">
         <v>1484</v>
       </c>
-      <c r="D60" s="1" t="n">
+      <c r="D60" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A60,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E60" s="1" t="n">
+      <c r="E60" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C60,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D60)</f>
         <v>1</v>
       </c>
-      <c r="F60" s="1" t="n">
+      <c r="F60" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C60,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D60)</f>
         <v>5</v>
       </c>
-      <c r="G60" s="1" t="n">
+      <c r="G60" s="0" t="n">
         <f aca="false">IF($D60=0,0,$E60/$D60)</f>
         <v>0.166666666666667</v>
       </c>
-      <c r="H60" s="1" t="n">
+      <c r="H60" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C60)</f>
         <v>18</v>
       </c>
-      <c r="I60" s="1" t="str">
+      <c r="I60" s="0" t="str">
         <f aca="false">IF(AND($D60&gt;0,$H60=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1" t="s">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B61" s="1" t="str">
+      <c r="B61" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A61,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C61" s="3" t="s">
-        <v>1482</v>
-      </c>
-      <c r="D61" s="1" t="n">
+      <c r="C61" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D61" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A61,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E61" s="1" t="n">
+      <c r="E61" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C61,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D61)</f>
         <v>1</v>
       </c>
-      <c r="F61" s="1" t="n">
+      <c r="F61" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C61,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D61)</f>
         <v>5</v>
       </c>
-      <c r="G61" s="1" t="n">
+      <c r="G61" s="0" t="n">
         <f aca="false">IF($D61=0,0,$E61/$D61)</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="H61" s="1" t="n">
+      <c r="H61" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C61)</f>
         <v>6</v>
       </c>
-      <c r="I61" s="1" t="str">
+      <c r="I61" s="0" t="str">
         <f aca="false">IF(AND($D61&gt;0,$H61=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="s">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B62" s="1" t="str">
+      <c r="B62" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A62,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="13" t="s">
         <v>1481</v>
       </c>
-      <c r="D62" s="1" t="n">
+      <c r="D62" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A62,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E62" s="1" t="n">
+      <c r="E62" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C62,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D62)</f>
         <v>2</v>
       </c>
-      <c r="F62" s="1" t="n">
+      <c r="F62" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C62,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D62)</f>
         <v>5</v>
       </c>
-      <c r="G62" s="1" t="n">
+      <c r="G62" s="0" t="n">
         <f aca="false">IF($D62=0,0,$E62/$D62)</f>
         <v>0.285714285714286</v>
       </c>
-      <c r="H62" s="1" t="n">
+      <c r="H62" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C62)</f>
         <v>17</v>
       </c>
-      <c r="I62" s="1" t="str">
+      <c r="I62" s="0" t="str">
         <f aca="false">IF(AND($D62&gt;0,$H62=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1" t="s">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B63" s="1" t="str">
+      <c r="B63" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A63,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C63" s="3" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D63" s="1" t="n">
+      <c r="C63" s="13" t="s">
+        <v>1852</v>
+      </c>
+      <c r="D63" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A63,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>15</v>
       </c>
-      <c r="E63" s="1" t="n">
+      <c r="E63" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C63,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D63)</f>
         <v>6</v>
       </c>
-      <c r="F63" s="1" t="n">
+      <c r="F63" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C63,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D63)</f>
         <v>9</v>
       </c>
-      <c r="G63" s="1" t="n">
+      <c r="G63" s="0" t="n">
         <f aca="false">IF($D63=0,0,$E63/$D63)</f>
         <v>0.4</v>
       </c>
-      <c r="H63" s="1" t="n">
+      <c r="H63" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C63)</f>
         <v>26</v>
       </c>
-      <c r="I63" s="1" t="str">
+      <c r="I63" s="0" t="str">
         <f aca="false">IF(AND($D63&gt;0,$H63=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="1" t="s">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B64" s="1" t="str">
+      <c r="B64" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A64,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C64" s="3" t="s">
-        <v>1488</v>
-      </c>
-      <c r="D64" s="1" t="n">
+      <c r="C64" s="13" t="s">
+        <v>1853</v>
+      </c>
+      <c r="D64" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A64,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>20</v>
       </c>
-      <c r="E64" s="1" t="n">
+      <c r="E64" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C64,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D64)</f>
         <v>10</v>
       </c>
-      <c r="F64" s="1" t="n">
+      <c r="F64" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C64,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D64)</f>
         <v>10</v>
       </c>
-      <c r="G64" s="1" t="n">
+      <c r="G64" s="0" t="n">
         <f aca="false">IF($D64=0,0,$E64/$D64)</f>
         <v>0.5</v>
       </c>
-      <c r="H64" s="1" t="n">
+      <c r="H64" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C64)</f>
         <v>40</v>
       </c>
-      <c r="I64" s="1" t="str">
+      <c r="I64" s="0" t="str">
         <f aca="false">IF(AND($D64&gt;0,$H64=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="1" t="s">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B65" s="1" t="str">
+      <c r="B65" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A65,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="13" t="s">
         <v>1495</v>
       </c>
-      <c r="D65" s="1" t="n">
+      <c r="D65" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A65,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E65" s="1" t="n">
+      <c r="E65" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C65,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D65)</f>
         <v>0</v>
       </c>
-      <c r="F65" s="1" t="n">
+      <c r="F65" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C65,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D65)</f>
         <v>0</v>
       </c>
-      <c r="G65" s="1" t="n">
+      <c r="G65" s="0" t="n">
         <f aca="false">IF($D65=0,0,$E65/$D65)</f>
         <v>0</v>
       </c>
-      <c r="H65" s="1" t="n">
+      <c r="H65" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C65)</f>
         <v>11</v>
       </c>
-      <c r="I65" s="1" t="str">
+      <c r="I65" s="0" t="str">
         <f aca="false">IF(AND($D65&gt;0,$H65=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1" t="s">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0" t="s">
         <v>1840</v>
       </c>
-      <c r="B66" s="1" t="str">
+      <c r="B66" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A66,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C66" s="3" t="s">
-        <v>1496</v>
-      </c>
-      <c r="D66" s="1" t="n">
+      <c r="C66" s="13" t="s">
+        <v>1854</v>
+      </c>
+      <c r="D66" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A66,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E66" s="1" t="n">
+      <c r="E66" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C66,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D66)</f>
         <v>0</v>
       </c>
-      <c r="F66" s="1" t="n">
+      <c r="F66" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C66,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D66)</f>
         <v>0</v>
       </c>
-      <c r="G66" s="1" t="n">
+      <c r="G66" s="0" t="n">
         <f aca="false">IF($D66=0,0,$E66/$D66)</f>
         <v>0</v>
       </c>
-      <c r="H66" s="1" t="n">
+      <c r="H66" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C66)</f>
         <v>20</v>
       </c>
-      <c r="I66" s="1" t="str">
+      <c r="I66" s="0" t="str">
         <f aca="false">IF(AND($D66&gt;0,$H66=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B67" s="1" t="str">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B67" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A67,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C67" s="13" t="s">
         <v>1474</v>
       </c>
-      <c r="D67" s="1" t="n">
+      <c r="D67" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A67,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>25</v>
       </c>
-      <c r="E67" s="1" t="n">
+      <c r="E67" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C67,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D67)</f>
         <v>4</v>
       </c>
-      <c r="F67" s="1" t="n">
+      <c r="F67" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C67,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D67)</f>
         <v>21</v>
       </c>
-      <c r="G67" s="1" t="n">
+      <c r="G67" s="0" t="n">
         <f aca="false">IF($D67=0,0,$E67/$D67)</f>
         <v>0.16</v>
       </c>
-      <c r="H67" s="1" t="n">
+      <c r="H67" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C67)</f>
         <v>36</v>
       </c>
-      <c r="I67" s="1" t="str">
+      <c r="I67" s="0" t="str">
         <f aca="false">IF(AND($D67&gt;0,$H67=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B68" s="1" t="str">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B68" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A68,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C68" s="13" t="s">
         <v>1480</v>
       </c>
-      <c r="D68" s="1" t="n">
+      <c r="D68" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A68,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E68" s="1" t="n">
+      <c r="E68" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C68,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D68)</f>
         <v>0</v>
       </c>
-      <c r="F68" s="1" t="n">
+      <c r="F68" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C68,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D68)</f>
         <v>7</v>
       </c>
-      <c r="G68" s="1" t="n">
+      <c r="G68" s="0" t="n">
         <f aca="false">IF($D68=0,0,$E68/$D68)</f>
         <v>0</v>
       </c>
-      <c r="H68" s="1" t="n">
+      <c r="H68" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C68)</f>
         <v>9</v>
       </c>
-      <c r="I68" s="1" t="str">
+      <c r="I68" s="0" t="str">
         <f aca="false">IF(AND($D68&gt;0,$H68=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B69" s="1" t="str">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B69" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A69,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C69" s="3" t="s">
-        <v>1479</v>
-      </c>
-      <c r="D69" s="1" t="n">
+      <c r="C69" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D69" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A69,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E69" s="1" t="n">
+      <c r="E69" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C69,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D69)</f>
         <v>0</v>
       </c>
-      <c r="F69" s="1" t="n">
+      <c r="F69" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C69,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D69)</f>
         <v>7</v>
       </c>
-      <c r="G69" s="1" t="n">
+      <c r="G69" s="0" t="n">
         <f aca="false">IF($D69=0,0,$E69/$D69)</f>
         <v>0</v>
       </c>
-      <c r="H69" s="1" t="n">
+      <c r="H69" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C69)</f>
         <v>11</v>
       </c>
-      <c r="I69" s="1" t="str">
+      <c r="I69" s="0" t="str">
         <f aca="false">IF(AND($D69&gt;0,$H69=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B70" s="1" t="str">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B70" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A70,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="13" t="s">
         <v>1491</v>
       </c>
-      <c r="D70" s="1" t="n">
+      <c r="D70" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A70,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>11</v>
       </c>
-      <c r="E70" s="1" t="n">
+      <c r="E70" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C70,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D70)</f>
         <v>2</v>
       </c>
-      <c r="F70" s="1" t="n">
+      <c r="F70" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C70,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D70)</f>
         <v>8</v>
       </c>
-      <c r="G70" s="1" t="n">
+      <c r="G70" s="0" t="n">
         <f aca="false">IF($D70=0,0,$E70/$D70)</f>
         <v>0.181818181818182</v>
       </c>
-      <c r="H70" s="1" t="n">
+      <c r="H70" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C70)</f>
         <v>10</v>
       </c>
-      <c r="I70" s="1" t="str">
+      <c r="I70" s="0" t="str">
         <f aca="false">IF(AND($D70&gt;0,$H70=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B71" s="1" t="str">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B71" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A71,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C71" s="13" t="s">
         <v>1490</v>
       </c>
-      <c r="D71" s="1" t="n">
+      <c r="D71" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A71,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>6</v>
       </c>
-      <c r="E71" s="1" t="n">
+      <c r="E71" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C71,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D71)</f>
         <v>2</v>
       </c>
-      <c r="F71" s="1" t="n">
+      <c r="F71" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C71,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D71)</f>
         <v>4</v>
       </c>
-      <c r="G71" s="1" t="n">
+      <c r="G71" s="0" t="n">
         <f aca="false">IF($D71=0,0,$E71/$D71)</f>
         <v>0.333333333333333</v>
       </c>
-      <c r="H71" s="1" t="n">
+      <c r="H71" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C71)</f>
         <v>20</v>
       </c>
-      <c r="I71" s="1" t="str">
+      <c r="I71" s="0" t="str">
         <f aca="false">IF(AND($D71&gt;0,$H71=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B72" s="1" t="str">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B72" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A72,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C72" s="13" t="s">
         <v>1477</v>
       </c>
-      <c r="D72" s="1" t="n">
+      <c r="D72" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A72,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>10</v>
       </c>
-      <c r="E72" s="1" t="n">
+      <c r="E72" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C72,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D72)</f>
         <v>5</v>
       </c>
-      <c r="F72" s="1" t="n">
+      <c r="F72" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C72,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D72)</f>
         <v>5</v>
       </c>
-      <c r="G72" s="1" t="n">
+      <c r="G72" s="0" t="n">
         <f aca="false">IF($D72=0,0,$E72/$D72)</f>
         <v>0.5</v>
       </c>
-      <c r="H72" s="1" t="n">
+      <c r="H72" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C72)</f>
         <v>20</v>
       </c>
-      <c r="I72" s="1" t="str">
+      <c r="I72" s="0" t="str">
         <f aca="false">IF(AND($D72&gt;0,$H72=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B73" s="1" t="str">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B73" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A73,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C73" s="3" t="s">
+      <c r="C73" s="13" t="s">
         <v>1484</v>
       </c>
-      <c r="D73" s="1" t="n">
+      <c r="D73" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A73,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E73" s="1" t="n">
+      <c r="E73" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C73,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D73)</f>
         <v>1</v>
       </c>
-      <c r="F73" s="1" t="n">
+      <c r="F73" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C73,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D73)</f>
         <v>6</v>
       </c>
-      <c r="G73" s="1" t="n">
+      <c r="G73" s="0" t="n">
         <f aca="false">IF($D73=0,0,$E73/$D73)</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="H73" s="1" t="n">
+      <c r="H73" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C73)</f>
         <v>18</v>
       </c>
-      <c r="I73" s="1" t="str">
+      <c r="I73" s="0" t="str">
         <f aca="false">IF(AND($D73&gt;0,$H73=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B74" s="1" t="str">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B74" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A74,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C74" s="3" t="s">
-        <v>1482</v>
-      </c>
-      <c r="D74" s="1" t="n">
+      <c r="C74" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D74" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A74,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>5</v>
       </c>
-      <c r="E74" s="1" t="n">
+      <c r="E74" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C74,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D74)</f>
         <v>1</v>
       </c>
-      <c r="F74" s="1" t="n">
+      <c r="F74" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C74,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D74)</f>
         <v>4</v>
       </c>
-      <c r="G74" s="1" t="n">
+      <c r="G74" s="0" t="n">
         <f aca="false">IF($D74=0,0,$E74/$D74)</f>
         <v>0.2</v>
       </c>
-      <c r="H74" s="1" t="n">
+      <c r="H74" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C74)</f>
         <v>6</v>
       </c>
-      <c r="I74" s="1" t="str">
+      <c r="I74" s="0" t="str">
         <f aca="false">IF(AND($D74&gt;0,$H74=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B75" s="1" t="str">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B75" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A75,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C75" s="3" t="s">
+      <c r="C75" s="13" t="s">
         <v>1481</v>
       </c>
-      <c r="D75" s="1" t="n">
+      <c r="D75" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A75,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>7</v>
       </c>
-      <c r="E75" s="1" t="n">
+      <c r="E75" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C75,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D75)</f>
         <v>2</v>
       </c>
-      <c r="F75" s="1" t="n">
+      <c r="F75" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C75,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D75)</f>
         <v>5</v>
       </c>
-      <c r="G75" s="1" t="n">
+      <c r="G75" s="0" t="n">
         <f aca="false">IF($D75=0,0,$E75/$D75)</f>
         <v>0.285714285714286</v>
       </c>
-      <c r="H75" s="1" t="n">
+      <c r="H75" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C75)</f>
         <v>17</v>
       </c>
-      <c r="I75" s="1" t="str">
+      <c r="I75" s="0" t="str">
         <f aca="false">IF(AND($D75&gt;0,$H75=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B76" s="1" t="str">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B76" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A76,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C76" s="3" t="s">
-        <v>1489</v>
-      </c>
-      <c r="D76" s="1" t="n">
+      <c r="C76" s="13" t="s">
+        <v>1852</v>
+      </c>
+      <c r="D76" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A76,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>13</v>
       </c>
-      <c r="E76" s="1" t="n">
+      <c r="E76" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C76,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D76)</f>
         <v>6</v>
       </c>
-      <c r="F76" s="1" t="n">
+      <c r="F76" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C76,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D76)</f>
         <v>7</v>
       </c>
-      <c r="G76" s="1" t="n">
+      <c r="G76" s="0" t="n">
         <f aca="false">IF($D76=0,0,$E76/$D76)</f>
         <v>0.461538461538462</v>
       </c>
-      <c r="H76" s="1" t="n">
+      <c r="H76" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C76)</f>
         <v>26</v>
       </c>
-      <c r="I76" s="1" t="str">
+      <c r="I76" s="0" t="str">
         <f aca="false">IF(AND($D76&gt;0,$H76=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B77" s="1" t="str">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B77" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A77,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C77" s="3" t="s">
-        <v>1488</v>
-      </c>
-      <c r="D77" s="1" t="n">
+      <c r="C77" s="13" t="s">
+        <v>1853</v>
+      </c>
+      <c r="D77" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A77,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>22</v>
       </c>
-      <c r="E77" s="1" t="n">
+      <c r="E77" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C77,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D77)</f>
         <v>11</v>
       </c>
-      <c r="F77" s="1" t="n">
+      <c r="F77" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C77,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D77)</f>
         <v>11</v>
       </c>
-      <c r="G77" s="1" t="n">
+      <c r="G77" s="0" t="n">
         <f aca="false">IF($D77=0,0,$E77/$D77)</f>
         <v>0.5</v>
       </c>
-      <c r="H77" s="1" t="n">
+      <c r="H77" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C77)</f>
         <v>40</v>
       </c>
-      <c r="I77" s="1" t="str">
+      <c r="I77" s="0" t="str">
         <f aca="false">IF(AND($D77&gt;0,$H77=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B78" s="1" t="str">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B78" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A78,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C78" s="13" t="s">
         <v>1495</v>
       </c>
-      <c r="D78" s="1" t="n">
+      <c r="D78" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A78,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E78" s="1" t="n">
+      <c r="E78" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C78,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D78)</f>
         <v>0</v>
       </c>
-      <c r="F78" s="1" t="n">
+      <c r="F78" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C78,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D78)</f>
         <v>0</v>
       </c>
-      <c r="G78" s="1" t="n">
+      <c r="G78" s="0" t="n">
         <f aca="false">IF($D78=0,0,$E78/$D78)</f>
         <v>0</v>
       </c>
-      <c r="H78" s="1" t="n">
+      <c r="H78" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C78)</f>
         <v>11</v>
       </c>
-      <c r="I78" s="1" t="str">
+      <c r="I78" s="0" t="str">
         <f aca="false">IF(AND($D78&gt;0,$H78=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="3" t="s">
-        <v>1842</v>
-      </c>
-      <c r="B79" s="1" t="str">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="13" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B79" s="0" t="str">
         <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A79,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>2026-10-27</v>
       </c>
-      <c r="C79" s="3" t="s">
-        <v>1496</v>
-      </c>
-      <c r="D79" s="1" t="n">
+      <c r="C79" s="13" t="s">
+        <v>1854</v>
+      </c>
+      <c r="D79" s="0" t="n">
         <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A79,'סקרים לפי ערוץ'!$A:$A,0))</f>
         <v>0</v>
       </c>
-      <c r="E79" s="1" t="n">
+      <c r="E79" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C79,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D79)</f>
         <v>0</v>
       </c>
-      <c r="F79" s="1" t="n">
+      <c r="F79" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C79,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D79)</f>
         <v>0</v>
       </c>
-      <c r="G79" s="1" t="n">
+      <c r="G79" s="0" t="n">
         <f aca="false">IF($D79=0,0,$E79/$D79)</f>
         <v>0</v>
       </c>
-      <c r="H79" s="1" t="n">
+      <c r="H79" s="0" t="n">
         <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C79)</f>
         <v>20</v>
       </c>
-      <c r="I79" s="1" t="str">
+      <c r="I79" s="0" t="str">
         <f aca="false">IF(AND($D79&gt;0,$H79=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B80" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A80,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C80" s="13" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D80" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!E:E,MATCH($A80,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>28</v>
+      </c>
+      <c r="E80" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C80,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D80)</f>
+        <v>4</v>
+      </c>
+      <c r="F80" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C80,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D80)</f>
+        <v>24</v>
+      </c>
+      <c r="G80" s="0" t="n">
+        <f aca="false">IF($D80=0,0,$E80/$D80)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H80" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C80)</f>
+        <v>36</v>
+      </c>
+      <c r="I80" s="0" t="str">
+        <f aca="false">IF(AND($D80&gt;0,$H80=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B81" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A81,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C81" s="13" t="s">
+        <v>1480</v>
+      </c>
+      <c r="D81" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!F:F,MATCH($A81,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E81" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C81,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D81)</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C81,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D81)</f>
+        <v>6</v>
+      </c>
+      <c r="G81" s="0" t="n">
+        <f aca="false">IF($D81=0,0,$E81/$D81)</f>
+        <v>0</v>
+      </c>
+      <c r="H81" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C81)</f>
+        <v>9</v>
+      </c>
+      <c r="I81" s="0" t="str">
+        <f aca="false">IF(AND($D81&gt;0,$H81=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B82" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A82,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C82" s="13" t="s">
+        <v>1850</v>
+      </c>
+      <c r="D82" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!G:G,MATCH($A82,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E82" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C82,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D82)</f>
+        <v>0</v>
+      </c>
+      <c r="F82" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C82,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D82)</f>
+        <v>7</v>
+      </c>
+      <c r="G82" s="0" t="n">
+        <f aca="false">IF($D82=0,0,$E82/$D82)</f>
+        <v>0</v>
+      </c>
+      <c r="H82" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C82)</f>
+        <v>11</v>
+      </c>
+      <c r="I82" s="0" t="str">
+        <f aca="false">IF(AND($D82&gt;0,$H82=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B83" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A83,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C83" s="13" t="s">
+        <v>1491</v>
+      </c>
+      <c r="D83" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!H:H,MATCH($A83,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>11</v>
+      </c>
+      <c r="E83" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C83,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D83)</f>
+        <v>2</v>
+      </c>
+      <c r="F83" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C83,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D83)</f>
+        <v>8</v>
+      </c>
+      <c r="G83" s="0" t="n">
+        <f aca="false">IF($D83=0,0,$E83/$D83)</f>
+        <v>0.181818181818182</v>
+      </c>
+      <c r="H83" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C83)</f>
+        <v>10</v>
+      </c>
+      <c r="I83" s="0" t="str">
+        <f aca="false">IF(AND($D83&gt;0,$H83=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B84" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A84,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C84" s="13" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D84" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!I:I,MATCH($A84,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>5</v>
+      </c>
+      <c r="E84" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C84,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D84)</f>
+        <v>2</v>
+      </c>
+      <c r="F84" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C84,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D84)</f>
+        <v>3</v>
+      </c>
+      <c r="G84" s="0" t="n">
+        <f aca="false">IF($D84=0,0,$E84/$D84)</f>
+        <v>0.4</v>
+      </c>
+      <c r="H84" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C84)</f>
+        <v>20</v>
+      </c>
+      <c r="I84" s="0" t="str">
+        <f aca="false">IF(AND($D84&gt;0,$H84=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B85" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A85,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C85" s="13" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D85" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!J:J,MATCH($A85,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>9</v>
+      </c>
+      <c r="E85" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C85,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D85)</f>
+        <v>4</v>
+      </c>
+      <c r="F85" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C85,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D85)</f>
+        <v>5</v>
+      </c>
+      <c r="G85" s="0" t="n">
+        <f aca="false">IF($D85=0,0,$E85/$D85)</f>
+        <v>0.444444444444444</v>
+      </c>
+      <c r="H85" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C85)</f>
+        <v>20</v>
+      </c>
+      <c r="I85" s="0" t="str">
+        <f aca="false">IF(AND($D85&gt;0,$H85=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B86" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A86,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C86" s="13" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D86" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!K:K,MATCH($A86,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E86" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C86,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D86)</f>
+        <v>1</v>
+      </c>
+      <c r="F86" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C86,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D86)</f>
+        <v>5</v>
+      </c>
+      <c r="G86" s="0" t="n">
+        <f aca="false">IF($D86=0,0,$E86/$D86)</f>
+        <v>0.166666666666667</v>
+      </c>
+      <c r="H86" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C86)</f>
+        <v>18</v>
+      </c>
+      <c r="I86" s="0" t="str">
+        <f aca="false">IF(AND($D86&gt;0,$H86=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B87" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A87,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C87" s="13" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D87" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!L:L,MATCH($A87,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>7</v>
+      </c>
+      <c r="E87" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C87,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D87)</f>
+        <v>1</v>
+      </c>
+      <c r="F87" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C87,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D87)</f>
+        <v>5</v>
+      </c>
+      <c r="G87" s="0" t="n">
+        <f aca="false">IF($D87=0,0,$E87/$D87)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="H87" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C87)</f>
+        <v>6</v>
+      </c>
+      <c r="I87" s="0" t="str">
+        <f aca="false">IF(AND($D87&gt;0,$H87=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B88" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A88,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C88" s="13" t="s">
+        <v>1481</v>
+      </c>
+      <c r="D88" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!M:M,MATCH($A88,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>6</v>
+      </c>
+      <c r="E88" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C88,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D88)</f>
+        <v>2</v>
+      </c>
+      <c r="F88" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C88,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D88)</f>
+        <v>4</v>
+      </c>
+      <c r="G88" s="0" t="n">
+        <f aca="false">IF($D88=0,0,$E88/$D88)</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="H88" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C88)</f>
+        <v>17</v>
+      </c>
+      <c r="I88" s="0" t="str">
+        <f aca="false">IF(AND($D88&gt;0,$H88=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B89" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A89,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C89" s="13" t="s">
+        <v>1852</v>
+      </c>
+      <c r="D89" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!N:N,MATCH($A89,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>13</v>
+      </c>
+      <c r="E89" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C89,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D89)</f>
+        <v>6</v>
+      </c>
+      <c r="F89" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C89,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D89)</f>
+        <v>7</v>
+      </c>
+      <c r="G89" s="0" t="n">
+        <f aca="false">IF($D89=0,0,$E89/$D89)</f>
+        <v>0.461538461538462</v>
+      </c>
+      <c r="H89" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C89)</f>
+        <v>26</v>
+      </c>
+      <c r="I89" s="0" t="str">
+        <f aca="false">IF(AND($D89&gt;0,$H89=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B90" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A90,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C90" s="13" t="s">
+        <v>1853</v>
+      </c>
+      <c r="D90" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!O:O,MATCH($A90,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>21</v>
+      </c>
+      <c r="E90" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C90,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D90)</f>
+        <v>11</v>
+      </c>
+      <c r="F90" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C90,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D90)</f>
+        <v>10</v>
+      </c>
+      <c r="G90" s="0" t="n">
+        <f aca="false">IF($D90=0,0,$E90/$D90)</f>
+        <v>0.523809523809524</v>
+      </c>
+      <c r="H90" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C90)</f>
+        <v>40</v>
+      </c>
+      <c r="I90" s="0" t="str">
+        <f aca="false">IF(AND($D90&gt;0,$H90=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B91" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A91,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C91" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="D91" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!P:P,MATCH($A91,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E91" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C91,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D91)</f>
+        <v>0</v>
+      </c>
+      <c r="F91" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C91,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D91)</f>
+        <v>0</v>
+      </c>
+      <c r="G91" s="0" t="n">
+        <f aca="false">IF($D91=0,0,$E91/$D91)</f>
+        <v>0</v>
+      </c>
+      <c r="H91" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C91)</f>
+        <v>11</v>
+      </c>
+      <c r="I91" s="0" t="str">
+        <f aca="false">IF(AND($D91&gt;0,$H91=0),"אין נתוני מועמדים לחישוב","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="13" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B92" s="0" t="str">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!$B:$B,MATCH($A92,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>2026-10-27</v>
+      </c>
+      <c r="C92" s="13" t="s">
+        <v>1854</v>
+      </c>
+      <c r="D92" s="0" t="n">
+        <f aca="false">INDEX('סקרים לפי ערוץ'!Q:Q,MATCH($A92,'סקרים לפי ערוץ'!$A:$A,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E92" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C92,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D92)</f>
+        <v>0</v>
+      </c>
+      <c r="F92" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C92,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;$D92)</f>
+        <v>0</v>
+      </c>
+      <c r="G92" s="0" t="n">
+        <f aca="false">IF($D92=0,0,$E92/$D92)</f>
+        <v>0</v>
+      </c>
+      <c r="H92" s="0" t="n">
+        <f aca="false">COUNTIFS('מועמדים 2026'!$A:$A,$C92)</f>
+        <v>20</v>
+      </c>
+      <c r="I92" s="0" t="str">
+        <f aca="false">IF(AND($D92&gt;0,$H92=0),"אין נתוני מועמדים לחישוב","")</f>
         <v/>
       </c>
     </row>

</xml_diff>